<commit_message>
modificaciones a la red neuronal y resultados
</commit_message>
<xml_diff>
--- a/02_outputs/model_registry.xlsx
+++ b/02_outputs/model_registry.xlsx
@@ -425,16 +425,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:AJ3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
@@ -450,6 +450,20 @@
     <col width="37" customWidth="1" min="20" max="20"/>
     <col width="60" customWidth="1" min="21" max="21"/>
     <col width="17" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
+    <col width="12" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+    <col width="13" customWidth="1" min="27" max="27"/>
+    <col width="15" customWidth="1" min="28" max="28"/>
+    <col width="10" customWidth="1" min="29" max="29"/>
+    <col width="7" customWidth="1" min="30" max="30"/>
+    <col width="47" customWidth="1" min="31" max="31"/>
+    <col width="46" customWidth="1" min="32" max="32"/>
+    <col width="8" customWidth="1" min="33" max="33"/>
+    <col width="16" customWidth="1" min="34" max="34"/>
+    <col width="22" customWidth="1" min="35" max="35"/>
+    <col width="8" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -563,6 +577,76 @@
           <t>sesgo_delta_log</t>
         </is>
       </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>n_params</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>epochs_run</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>cv_mae_log</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>cv_mae_cop_M</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>esp_mae_log</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>esp_mae_cop_M</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>l1_ratio</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>features_grupos</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>arquitectura</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>reg_l2</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>early_stopping</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>reg_l1_l2</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>device</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -640,6 +724,124 @@
       </c>
       <c r="V2" t="n">
         <v>0.01858</v>
+      </c>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NN_002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Jonathan</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>NeuralNetwork_PyTorch</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>29</v>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>val_split=0.2</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="n">
+        <v>0.20457</v>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>5x5</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>submission_NN_002_ep75_p48k.csv</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>MLP PyTorch 256→128→64→1 con ReLU, Dropout y Elastic Net. Backend: mps. l1=0.0001, l2=0.0001 (weight_decay). EarlyStopping patience=15. Épocas efectivas: 75/200. MAE_log val.interno=0.21823 (optimista). MAE_log CV espacial=0.24954 (honesto). Sesgo Δ=+0.03131.</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="n">
+        <v>48897</v>
+      </c>
+      <c r="X3" t="n">
+        <v>75</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>0.21823</v>
+      </c>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="n">
+        <v>0.24954</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>170.23</v>
+      </c>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>structural=7, text=11, osm=10, es_apartamento</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>p→256(Drop0.3)→128(Drop0.2)→64→1 (ReLU, MPS)</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>patience=15</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>l1=0.0001, l2=0.0001</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>mps</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Estandarizar nomenclatura 06_ en red neuronal: script, outputs y registry
Renombra MODEL_ID de NN_002 a 06_NN para alinear con el prefijo del script
06_neural_network_pytorch.py. Actualiza carpeta de outputs, submission y
model_registry.xlsx.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02_outputs/model_registry.xlsx
+++ b/02_outputs/model_registry.xlsx
@@ -845,7 +845,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NN_002</t>
+          <t>06_NN</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -892,7 +892,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>submission_NN_002_ep75_p48k.csv</t>
+          <t>submission_06_NN_ep75_p48k.csv</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">

</xml_diff>

<commit_message>
feat: run CART_001 and CART_002 - add outputs and submissions
</commit_message>
<xml_diff>
--- a/02_outputs/model_registry.xlsx
+++ b/02_outputs/model_registry.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="registry" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="registry" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ9"/>
+  <dimension ref="A1:AR11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -459,222 +471,228 @@
     <col width="18" customWidth="1" min="41" max="41"/>
     <col width="14" customWidth="1" min="42" max="42"/>
     <col width="13" customWidth="1" min="43" max="43"/>
+    <col width="11" customWidth="1" min="44" max="44"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>model_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>fecha</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>autor</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>algoritmo</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>n_features</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>n_coefs_nonzero</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>cv_folds</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>rand_cv_mae_log</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>rand_cv_mae_cop_M</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>esp_cv_mae_log</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>esp_cv_mae_cop_M</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>sesgo_cv_delta_log</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>train_mae_log</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>kaggle_public_MAE</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>l1_ratio_spatial</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>alpha_spatial</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>l1_ratio_random</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>alpha_random</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>spatial_grid</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>submission_file</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>notas</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>sesgo_delta_log</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>n_params</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>cv_mae_log</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>cv_std_log</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>esp_mae_log</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>esp_std_log</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>l1_ratio</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>alpha</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>features_grupos</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>epochs_run</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>cv_mae_cop_M</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>esp_mae_cop_M</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>arquitectura</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>reg_l2</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>early_stopping</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>reg_l1_l2</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>device</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>n_estimators</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>max_depth</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>min_samples_leaf</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>max_features</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>sesgo_delta</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>ccp_alpha</t>
         </is>
       </c>
     </row>
@@ -776,6 +794,7 @@
       <c r="AO2" t="inlineStr"/>
       <c r="AP2" t="inlineStr"/>
       <c r="AQ2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -869,6 +888,7 @@
       <c r="AO3" t="inlineStr"/>
       <c r="AP3" t="inlineStr"/>
       <c r="AQ3" t="inlineStr"/>
+      <c r="AR3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -980,6 +1000,7 @@
       <c r="AO4" t="inlineStr"/>
       <c r="AP4" t="inlineStr"/>
       <c r="AQ4" t="inlineStr"/>
+      <c r="AR4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1081,6 +1102,7 @@
       <c r="AQ5" t="n">
         <v>0.02805</v>
       </c>
+      <c r="AR5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1182,6 +1204,7 @@
       <c r="AQ6" t="n">
         <v>0.10949</v>
       </c>
+      <c r="AR6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1285,6 +1308,7 @@
       <c r="AQ7" t="n">
         <v>0.05069</v>
       </c>
+      <c r="AR7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1388,6 +1412,7 @@
       <c r="AQ8" t="n">
         <v>0.04949</v>
       </c>
+      <c r="AR8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1477,10 +1502,8 @@
       <c r="AM9" t="n">
         <v>500</v>
       </c>
-      <c r="AN9" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
+      <c r="AN9" t="n">
+        <v>15</v>
       </c>
       <c r="AO9" t="n">
         <v>5</v>
@@ -1492,6 +1515,207 @@
       </c>
       <c r="AQ9" t="n">
         <v>0.07192</v>
+      </c>
+      <c r="AR9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CART_001</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Dani</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>8</v>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="n">
+        <v>5</v>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="n">
+        <v>0.19418</v>
+      </c>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>5x5</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>CART_dNone_leaf1_ccp00_cv5_CART_001.csv</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Baseline: solo features estructurales + es_apartamento. Defaults sklearn: depth=None, leaf=1, ccp=0. Sin OSM ni texto. Sesgo Δ=+0.03824.</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
+      <c r="X10" t="n">
+        <v>0.26502</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>0.00274</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>0.30326</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>structural=7, text=0, osm=0, es_apartamento</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr"/>
+      <c r="AG10" t="inlineStr"/>
+      <c r="AH10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr"/>
+      <c r="AJ10" t="inlineStr"/>
+      <c r="AK10" t="inlineStr"/>
+      <c r="AL10" t="inlineStr"/>
+      <c r="AM10" t="inlineStr"/>
+      <c r="AN10" t="inlineStr"/>
+      <c r="AO10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP10" t="inlineStr"/>
+      <c r="AQ10" t="n">
+        <v>0.03824</v>
+      </c>
+      <c r="AR10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CART_002</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Dani</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>29</v>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="n">
+        <v>5</v>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="n">
+        <v>0.22825</v>
+      </c>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>5x5</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>CART_d10_leaf20_ccp00001_cv5_CART_002.csv</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>All features: estructurales + OSM + texto. GridSearchCV espacial. Params: {'ccp_alpha': 0.0001, 'max_depth': 10, 'min_samples_leaf': 20}. Sesgo Delta=+0.04144.</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr"/>
+      <c r="X11" t="n">
+        <v>0.2326</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>0.00216</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>0.27405</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>0.01087</v>
+      </c>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr"/>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>structural=7, osm=10, text=11, es_apartamento</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr"/>
+      <c r="AG11" t="inlineStr"/>
+      <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr"/>
+      <c r="AJ11" t="inlineStr"/>
+      <c r="AK11" t="inlineStr"/>
+      <c r="AL11" t="inlineStr"/>
+      <c r="AM11" t="inlineStr"/>
+      <c r="AN11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AO11" t="n">
+        <v>20</v>
+      </c>
+      <c r="AP11" t="inlineStr"/>
+      <c r="AQ11" t="n">
+        <v>0.04144</v>
+      </c>
+      <c r="AR11" t="n">
+        <v>0.0001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
run all XGBoost models - add outputs and submissions
</commit_message>
<xml_diff>
--- a/02_outputs/model_registry.xlsx
+++ b/02_outputs/model_registry.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR11"/>
+  <dimension ref="A1:AZ15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -472,6 +472,14 @@
     <col width="14" customWidth="1" min="42" max="42"/>
     <col width="13" customWidth="1" min="43" max="43"/>
     <col width="11" customWidth="1" min="44" max="44"/>
+    <col width="15" customWidth="1" min="45" max="45"/>
+    <col width="11" customWidth="1" min="46" max="46"/>
+    <col width="18" customWidth="1" min="47" max="47"/>
+    <col width="18" customWidth="1" min="48" max="48"/>
+    <col width="8" customWidth="1" min="49" max="49"/>
+    <col width="12" customWidth="1" min="50" max="50"/>
+    <col width="11" customWidth="1" min="51" max="51"/>
+    <col width="15" customWidth="1" min="52" max="52"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -693,6 +701,46 @@
       <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>ccp_alpha</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>learning_rate</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>subsample</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>colsample_bytree</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>min_child_weight</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>gamma</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>reg_lambda</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>reg_alpha</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>n_iter_search</t>
         </is>
       </c>
     </row>
@@ -795,6 +843,14 @@
       <c r="AP2" t="inlineStr"/>
       <c r="AQ2" t="inlineStr"/>
       <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr"/>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr"/>
+      <c r="AX2" t="inlineStr"/>
+      <c r="AY2" t="inlineStr"/>
+      <c r="AZ2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -889,6 +945,14 @@
       <c r="AP3" t="inlineStr"/>
       <c r="AQ3" t="inlineStr"/>
       <c r="AR3" t="inlineStr"/>
+      <c r="AS3" t="inlineStr"/>
+      <c r="AT3" t="inlineStr"/>
+      <c r="AU3" t="inlineStr"/>
+      <c r="AV3" t="inlineStr"/>
+      <c r="AW3" t="inlineStr"/>
+      <c r="AX3" t="inlineStr"/>
+      <c r="AY3" t="inlineStr"/>
+      <c r="AZ3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1001,6 +1065,14 @@
       <c r="AP4" t="inlineStr"/>
       <c r="AQ4" t="inlineStr"/>
       <c r="AR4" t="inlineStr"/>
+      <c r="AS4" t="inlineStr"/>
+      <c r="AT4" t="inlineStr"/>
+      <c r="AU4" t="inlineStr"/>
+      <c r="AV4" t="inlineStr"/>
+      <c r="AW4" t="inlineStr"/>
+      <c r="AX4" t="inlineStr"/>
+      <c r="AY4" t="inlineStr"/>
+      <c r="AZ4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1103,6 +1175,14 @@
         <v>0.02805</v>
       </c>
       <c r="AR5" t="inlineStr"/>
+      <c r="AS5" t="inlineStr"/>
+      <c r="AT5" t="inlineStr"/>
+      <c r="AU5" t="inlineStr"/>
+      <c r="AV5" t="inlineStr"/>
+      <c r="AW5" t="inlineStr"/>
+      <c r="AX5" t="inlineStr"/>
+      <c r="AY5" t="inlineStr"/>
+      <c r="AZ5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1205,6 +1285,14 @@
         <v>0.10949</v>
       </c>
       <c r="AR6" t="inlineStr"/>
+      <c r="AS6" t="inlineStr"/>
+      <c r="AT6" t="inlineStr"/>
+      <c r="AU6" t="inlineStr"/>
+      <c r="AV6" t="inlineStr"/>
+      <c r="AW6" t="inlineStr"/>
+      <c r="AX6" t="inlineStr"/>
+      <c r="AY6" t="inlineStr"/>
+      <c r="AZ6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1309,6 +1397,14 @@
         <v>0.05069</v>
       </c>
       <c r="AR7" t="inlineStr"/>
+      <c r="AS7" t="inlineStr"/>
+      <c r="AT7" t="inlineStr"/>
+      <c r="AU7" t="inlineStr"/>
+      <c r="AV7" t="inlineStr"/>
+      <c r="AW7" t="inlineStr"/>
+      <c r="AX7" t="inlineStr"/>
+      <c r="AY7" t="inlineStr"/>
+      <c r="AZ7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1413,6 +1509,14 @@
         <v>0.04949</v>
       </c>
       <c r="AR8" t="inlineStr"/>
+      <c r="AS8" t="inlineStr"/>
+      <c r="AT8" t="inlineStr"/>
+      <c r="AU8" t="inlineStr"/>
+      <c r="AV8" t="inlineStr"/>
+      <c r="AW8" t="inlineStr"/>
+      <c r="AX8" t="inlineStr"/>
+      <c r="AY8" t="inlineStr"/>
+      <c r="AZ8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1517,6 +1621,14 @@
         <v>0.07192</v>
       </c>
       <c r="AR9" t="inlineStr"/>
+      <c r="AS9" t="inlineStr"/>
+      <c r="AT9" t="inlineStr"/>
+      <c r="AU9" t="inlineStr"/>
+      <c r="AV9" t="inlineStr"/>
+      <c r="AW9" t="inlineStr"/>
+      <c r="AX9" t="inlineStr"/>
+      <c r="AY9" t="inlineStr"/>
+      <c r="AZ9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1615,6 +1727,14 @@
       <c r="AR10" t="n">
         <v>0</v>
       </c>
+      <c r="AS10" t="inlineStr"/>
+      <c r="AT10" t="inlineStr"/>
+      <c r="AU10" t="inlineStr"/>
+      <c r="AV10" t="inlineStr"/>
+      <c r="AW10" t="inlineStr"/>
+      <c r="AX10" t="inlineStr"/>
+      <c r="AY10" t="inlineStr"/>
+      <c r="AZ10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1702,10 +1822,8 @@
       <c r="AK11" t="inlineStr"/>
       <c r="AL11" t="inlineStr"/>
       <c r="AM11" t="inlineStr"/>
-      <c r="AN11" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="AN11" t="n">
+        <v>10</v>
       </c>
       <c r="AO11" t="n">
         <v>20</v>
@@ -1716,6 +1834,472 @@
       </c>
       <c r="AR11" t="n">
         <v>0.0001</v>
+      </c>
+      <c r="AS11" t="inlineStr"/>
+      <c r="AT11" t="inlineStr"/>
+      <c r="AU11" t="inlineStr"/>
+      <c r="AV11" t="inlineStr"/>
+      <c r="AW11" t="inlineStr"/>
+      <c r="AX11" t="inlineStr"/>
+      <c r="AY11" t="inlineStr"/>
+      <c r="AZ11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>XGB_001</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Dani</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>8</v>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="n">
+        <v>5</v>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="n">
+        <v>0.23932</v>
+      </c>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>5x5</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>XGB_nest100_d6_lr03_cv5_XGB_001.csv</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Baseline: solo estructurales + es_apartamento. Defaults XGBoost: n_est=100, depth=6, lr=0.3. Sin OSM ni texto. Sesgo Delta=+0.02424.</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr"/>
+      <c r="X12" t="n">
+        <v>0.25235</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>0.00246</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>0.27659</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>0.01182</v>
+      </c>
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr"/>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>structural=7, text=0, osm=0, es_apartamento</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr"/>
+      <c r="AF12" t="inlineStr"/>
+      <c r="AG12" t="inlineStr"/>
+      <c r="AH12" t="inlineStr"/>
+      <c r="AI12" t="inlineStr"/>
+      <c r="AJ12" t="inlineStr"/>
+      <c r="AK12" t="inlineStr"/>
+      <c r="AL12" t="inlineStr"/>
+      <c r="AM12" t="n">
+        <v>100</v>
+      </c>
+      <c r="AN12" t="n">
+        <v>6</v>
+      </c>
+      <c r="AO12" t="inlineStr"/>
+      <c r="AP12" t="inlineStr"/>
+      <c r="AQ12" t="n">
+        <v>0.02424</v>
+      </c>
+      <c r="AR12" t="inlineStr"/>
+      <c r="AS12" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AT12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV12" t="inlineStr"/>
+      <c r="AW12" t="inlineStr"/>
+      <c r="AX12" t="inlineStr"/>
+      <c r="AY12" t="inlineStr"/>
+      <c r="AZ12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>XGB_002</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Dani</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>29</v>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="n">
+        <v>5</v>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="n">
+        <v>0.1391</v>
+      </c>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>5x5</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>XGB_nest100_d6_lr03_allfeats_cv5_XGB_002.csv</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>All features: estructurales + OSM + texto. Defaults XGBoost sin tuning. Sesgo Delta=+0.10189.</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr"/>
+      <c r="W13" t="inlineStr"/>
+      <c r="X13" t="n">
+        <v>0.1737</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>0.00133</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>0.2756</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>0.01177</v>
+      </c>
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr"/>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>structural=7, osm=10, text=11, es_apartamento</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr"/>
+      <c r="AF13" t="inlineStr"/>
+      <c r="AG13" t="inlineStr"/>
+      <c r="AH13" t="inlineStr"/>
+      <c r="AI13" t="inlineStr"/>
+      <c r="AJ13" t="inlineStr"/>
+      <c r="AK13" t="inlineStr"/>
+      <c r="AL13" t="inlineStr"/>
+      <c r="AM13" t="n">
+        <v>100</v>
+      </c>
+      <c r="AN13" t="n">
+        <v>6</v>
+      </c>
+      <c r="AO13" t="inlineStr"/>
+      <c r="AP13" t="inlineStr"/>
+      <c r="AQ13" t="n">
+        <v>0.10189</v>
+      </c>
+      <c r="AR13" t="inlineStr"/>
+      <c r="AS13" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AT13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV13" t="inlineStr"/>
+      <c r="AW13" t="inlineStr"/>
+      <c r="AX13" t="inlineStr"/>
+      <c r="AY13" t="inlineStr"/>
+      <c r="AZ13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>XGB_003</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Dani</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>29</v>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="n">
+        <v>5</v>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="n">
+        <v>0.14165</v>
+      </c>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>5x5</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>XGB_nest300_d7_lr005_cv5_XGB_003.csv</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>Depth tuning: GridSearch sobre max_depth y learning_rate. n_estimators fijo=300. Params: {'learning_rate': 0.05, 'max_depth': 7}. Sesgo Delta=+0.08760.</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="inlineStr"/>
+      <c r="X14" t="n">
+        <v>0.17131</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>0.00134</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>0.25891</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>0.00825</v>
+      </c>
+      <c r="AB14" t="inlineStr"/>
+      <c r="AC14" t="inlineStr"/>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>structural=7, osm=10, text=11, es_apartamento</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr"/>
+      <c r="AF14" t="inlineStr"/>
+      <c r="AG14" t="inlineStr"/>
+      <c r="AH14" t="inlineStr"/>
+      <c r="AI14" t="inlineStr"/>
+      <c r="AJ14" t="inlineStr"/>
+      <c r="AK14" t="inlineStr"/>
+      <c r="AL14" t="inlineStr"/>
+      <c r="AM14" t="n">
+        <v>300</v>
+      </c>
+      <c r="AN14" t="n">
+        <v>7</v>
+      </c>
+      <c r="AO14" t="inlineStr"/>
+      <c r="AP14" t="inlineStr"/>
+      <c r="AQ14" t="n">
+        <v>0.0876</v>
+      </c>
+      <c r="AR14" t="inlineStr"/>
+      <c r="AS14" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="AT14" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AU14" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AV14" t="inlineStr"/>
+      <c r="AW14" t="inlineStr"/>
+      <c r="AX14" t="inlineStr"/>
+      <c r="AY14" t="inlineStr"/>
+      <c r="AZ14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>XGB_004</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Dani</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>29</v>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="n">
+        <v>5</v>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="n">
+        <v>0.18526</v>
+      </c>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>5x5</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>XGB_nest356_d6_lr0078_cv5_XGB_004.csv</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>Tuning exhaustivo: RandomizedSearchCV 50 iter, 9 hiperparametros, CV espacial. Params: {'colsample_bytree': 0.6356745158869479, 'gamma': 0.41436875457596467, 'learning_rate': 0.07778313207178196, 'max_depth': 6, 'min_child_weight': 9, 'n_estimators': 356, 'reg_alpha': 0.8021969807540397, 'reg_lambda': 0.8354778965589686, 'subsample': 0.9947547746402069}. Sesgo Delta=+0.06037.</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="inlineStr"/>
+      <c r="X15" t="n">
+        <v>0.19596</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>0.0019</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>0.25634</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>0.00665</v>
+      </c>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr"/>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>structural=7, osm=10, text=11, es_apartamento</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr"/>
+      <c r="AF15" t="inlineStr"/>
+      <c r="AG15" t="inlineStr"/>
+      <c r="AH15" t="inlineStr"/>
+      <c r="AI15" t="inlineStr"/>
+      <c r="AJ15" t="inlineStr"/>
+      <c r="AK15" t="inlineStr"/>
+      <c r="AL15" t="inlineStr"/>
+      <c r="AM15" t="n">
+        <v>356</v>
+      </c>
+      <c r="AN15" t="n">
+        <v>6</v>
+      </c>
+      <c r="AO15" t="inlineStr"/>
+      <c r="AP15" t="inlineStr"/>
+      <c r="AQ15" t="n">
+        <v>0.06037</v>
+      </c>
+      <c r="AR15" t="inlineStr"/>
+      <c r="AS15" t="n">
+        <v>0.07779999999999999</v>
+      </c>
+      <c r="AT15" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="AU15" t="n">
+        <v>0.636</v>
+      </c>
+      <c r="AV15" t="n">
+        <v>9</v>
+      </c>
+      <c r="AW15" t="n">
+        <v>0.4144</v>
+      </c>
+      <c r="AX15" t="n">
+        <v>0.8355</v>
+      </c>
+      <c r="AY15" t="n">
+        <v>0.8022</v>
+      </c>
+      <c r="AZ15" t="n">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
run XGB_005 spatial and XGB_006 more iter - add outputs
</commit_message>
<xml_diff>
--- a/02_outputs/model_registry.xlsx
+++ b/02_outputs/model_registry.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ15"/>
+  <dimension ref="A1:AZ17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -457,7 +457,7 @@
     <col width="13" customWidth="1" min="27" max="27"/>
     <col width="10" customWidth="1" min="28" max="28"/>
     <col width="7" customWidth="1" min="29" max="29"/>
-    <col width="47" customWidth="1" min="30" max="30"/>
+    <col width="60" customWidth="1" min="30" max="30"/>
     <col width="12" customWidth="1" min="31" max="31"/>
     <col width="14" customWidth="1" min="32" max="32"/>
     <col width="15" customWidth="1" min="33" max="33"/>
@@ -2302,6 +2302,242 @@
         <v>50</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>XGB_005</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>30</v>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="n">
+        <v>5</v>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="n">
+        <v>0.14478</v>
+      </c>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>5x5</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>XGB_spatial_nest304_d4_lr0014_cv5_XGB_005.csv</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>All features + target encoding espacial leave-one-out. RandomizedSearchCV 50 iter, CV espacial. Params: {'colsample_bytree': 0.6594878151468806, 'gamma': 0.4224376554847273, 'learning_rate': 0.014421667789806915, 'max_depth': 4, 'min_child_weight': 3, 'n_estimators': 304, 'reg_alpha': 0.4960374542934062, 'reg_lambda': 3.6180066141137273, 'subsample': 0.739334641781279}. Sesgo Delta=+0.14700.</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr"/>
+      <c r="X16" t="n">
+        <v>0.14821</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>0.00297</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>0.29521</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>0.02317</v>
+      </c>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr"/>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>structural=7, osm=10, text=11, target_espacial=1, es_apartamento</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr"/>
+      <c r="AF16" t="inlineStr"/>
+      <c r="AG16" t="inlineStr"/>
+      <c r="AH16" t="inlineStr"/>
+      <c r="AI16" t="inlineStr"/>
+      <c r="AJ16" t="inlineStr"/>
+      <c r="AK16" t="inlineStr"/>
+      <c r="AL16" t="inlineStr"/>
+      <c r="AM16" t="n">
+        <v>304</v>
+      </c>
+      <c r="AN16" t="n">
+        <v>4</v>
+      </c>
+      <c r="AO16" t="inlineStr"/>
+      <c r="AP16" t="inlineStr"/>
+      <c r="AQ16" t="n">
+        <v>0.147</v>
+      </c>
+      <c r="AR16" t="inlineStr"/>
+      <c r="AS16" t="n">
+        <v>0.0144</v>
+      </c>
+      <c r="AT16" t="n">
+        <v>0.739</v>
+      </c>
+      <c r="AU16" t="n">
+        <v>0.659</v>
+      </c>
+      <c r="AV16" t="n">
+        <v>3</v>
+      </c>
+      <c r="AW16" t="n">
+        <v>0.4224</v>
+      </c>
+      <c r="AX16" t="n">
+        <v>3.618</v>
+      </c>
+      <c r="AY16" t="n">
+        <v>0.496</v>
+      </c>
+      <c r="AZ16" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>XGB_006</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>29</v>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="n">
+        <v>5</v>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="n">
+        <v>0.16684</v>
+      </c>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>5x5</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>XGB_iter150_nest564_d8_lr0075_cv5_XGB_006.csv</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>All features. RandomizedSearchCV 150 iter (3x XGB_004). Mismo espacio de busqueda que XGB_004 para comparacion justa. Params: {'colsample_bytree': 0.8812293428703453, 'gamma': 0.43838281838087473, 'learning_rate': 0.07499553225602242, 'max_depth': 8, 'min_child_weight': 4, 'n_estimators': 564, 'reg_alpha': 0.12748866233198242, 'reg_lambda': 2.2877928075216527, 'subsample': 0.9189181463118214}. Sesgo Delta=+0.06906.</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="inlineStr"/>
+      <c r="X17" t="n">
+        <v>0.18619</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>0.00112</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>0.25525</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>0.00721</v>
+      </c>
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr"/>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>structural=7, osm=10, text=11, es_apartamento</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr"/>
+      <c r="AF17" t="inlineStr"/>
+      <c r="AG17" t="inlineStr"/>
+      <c r="AH17" t="inlineStr"/>
+      <c r="AI17" t="inlineStr"/>
+      <c r="AJ17" t="inlineStr"/>
+      <c r="AK17" t="inlineStr"/>
+      <c r="AL17" t="inlineStr"/>
+      <c r="AM17" t="n">
+        <v>564</v>
+      </c>
+      <c r="AN17" t="n">
+        <v>8</v>
+      </c>
+      <c r="AO17" t="inlineStr"/>
+      <c r="AP17" t="inlineStr"/>
+      <c r="AQ17" t="n">
+        <v>0.06906</v>
+      </c>
+      <c r="AR17" t="inlineStr"/>
+      <c r="AS17" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="AT17" t="n">
+        <v>0.919</v>
+      </c>
+      <c r="AU17" t="n">
+        <v>0.881</v>
+      </c>
+      <c r="AV17" t="n">
+        <v>4</v>
+      </c>
+      <c r="AW17" t="n">
+        <v>0.4384</v>
+      </c>
+      <c r="AX17" t="n">
+        <v>2.2878</v>
+      </c>
+      <c r="AY17" t="n">
+        <v>0.1275</v>
+      </c>
+      <c r="AZ17" t="n">
+        <v>150</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
prueba de mejoras al modelo de elastic net
</commit_message>
<xml_diff>
--- a/02_outputs/model_registry.xlsx
+++ b/02_outputs/model_registry.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="registry" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="registry" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ17"/>
+  <dimension ref="A1:AZ18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2538,6 +2538,114 @@
         <v>150</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>EN_002</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Jonathan</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>ElasticNet</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>37</v>
+      </c>
+      <c r="F18" t="n">
+        <v>17</v>
+      </c>
+      <c r="G18" t="n">
+        <v>5</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.26348</v>
+      </c>
+      <c r="I18" t="n">
+        <v>176.6</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.29778</v>
+      </c>
+      <c r="K18" t="n">
+        <v>199.13</v>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="n">
+        <v>0.2815</v>
+      </c>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="n">
+        <v>1</v>
+      </c>
+      <c r="P18" t="n">
+        <v>0.01935773</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>1</v>
+      </c>
+      <c r="R18" t="n">
+        <v>0.00033828</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>5x5</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>submission_EN_002_l1r100_a2en02.csv</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>EN_002: log-transforms + interacciones + poly espacial. CV aleatorio MAE_log=0.26348 (optimista). CV espacial  MAE_log=0.29778 (honesto). Sesgo Δ=+0.03430. Modelo final: l1_ratio=1.0, α=1.94e-02. 17/37 coefs≠0.</t>
+        </is>
+      </c>
+      <c r="V18" t="n">
+        <v>0.0343</v>
+      </c>
+      <c r="W18" t="inlineStr"/>
+      <c r="X18" t="inlineStr"/>
+      <c r="Y18" t="inlineStr"/>
+      <c r="Z18" t="inlineStr"/>
+      <c r="AA18" t="inlineStr"/>
+      <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr"/>
+      <c r="AD18" t="inlineStr"/>
+      <c r="AE18" t="inlineStr"/>
+      <c r="AF18" t="inlineStr"/>
+      <c r="AG18" t="inlineStr"/>
+      <c r="AH18" t="inlineStr"/>
+      <c r="AI18" t="inlineStr"/>
+      <c r="AJ18" t="inlineStr"/>
+      <c r="AK18" t="inlineStr"/>
+      <c r="AL18" t="inlineStr"/>
+      <c r="AM18" t="inlineStr"/>
+      <c r="AN18" t="inlineStr"/>
+      <c r="AO18" t="inlineStr"/>
+      <c r="AP18" t="inlineStr"/>
+      <c r="AQ18" t="inlineStr"/>
+      <c r="AR18" t="inlineStr"/>
+      <c r="AS18" t="inlineStr"/>
+      <c r="AT18" t="inlineStr"/>
+      <c r="AU18" t="inlineStr"/>
+      <c r="AV18" t="inlineStr"/>
+      <c r="AW18" t="inlineStr"/>
+      <c r="AX18" t="inlineStr"/>
+      <c r="AY18" t="inlineStr"/>
+      <c r="AZ18" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Prueba de mejoras al neural network
</commit_message>
<xml_diff>
--- a/02_outputs/model_registry.xlsx
+++ b/02_outputs/model_registry.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ18"/>
+  <dimension ref="A1:AZ19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -461,7 +461,7 @@
     <col width="12" customWidth="1" min="31" max="31"/>
     <col width="14" customWidth="1" min="32" max="32"/>
     <col width="15" customWidth="1" min="33" max="33"/>
-    <col width="46" customWidth="1" min="34" max="34"/>
+    <col width="60" customWidth="1" min="34" max="34"/>
     <col width="8" customWidth="1" min="35" max="35"/>
     <col width="16" customWidth="1" min="36" max="36"/>
     <col width="22" customWidth="1" min="37" max="37"/>
@@ -2646,6 +2646,126 @@
       <c r="AY18" t="inlineStr"/>
       <c r="AZ18" t="inlineStr"/>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>NN_003</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Jonathan</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>NeuralNetwork_PyTorch</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>37</v>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>val_split=0.2</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="n">
+        <v>0.13739</v>
+      </c>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>5x5</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>submission_NN_003_ep182_p118k.csv</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>NN_003: BN + 4 capas + features EN_002 + reg reducida + patience=30. Backend: mps. l1=5e-05, l2=5e-05. Épocas: 182/300. MAE_log val.interno=0.18910. MAE_log CV espacial=0.24331. Sesgo Δ=+0.05420.</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr"/>
+      <c r="W19" t="n">
+        <v>118145</v>
+      </c>
+      <c r="X19" t="n">
+        <v>0.1891</v>
+      </c>
+      <c r="Y19" t="inlineStr"/>
+      <c r="Z19" t="n">
+        <v>0.24331</v>
+      </c>
+      <c r="AA19" t="inlineStr"/>
+      <c r="AB19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr"/>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>structural=10, text=11, osm=10, spatial_poly=5, es_apartamento</t>
+        </is>
+      </c>
+      <c r="AE19" t="n">
+        <v>182</v>
+      </c>
+      <c r="AF19" t="inlineStr"/>
+      <c r="AG19" t="n">
+        <v>165.01</v>
+      </c>
+      <c r="AH19" t="inlineStr">
+        <is>
+          <t>p→256(BN,Drop0.2)→256(BN,Drop0.2)→128(BN,Drop0.1)→64(BN)→1 (ReLU)</t>
+        </is>
+      </c>
+      <c r="AI19" t="inlineStr"/>
+      <c r="AJ19" t="inlineStr">
+        <is>
+          <t>patience=30</t>
+        </is>
+      </c>
+      <c r="AK19" t="inlineStr">
+        <is>
+          <t>l1=5e-05, l2=5e-05</t>
+        </is>
+      </c>
+      <c r="AL19" t="inlineStr">
+        <is>
+          <t>mps</t>
+        </is>
+      </c>
+      <c r="AM19" t="inlineStr"/>
+      <c r="AN19" t="inlineStr"/>
+      <c r="AO19" t="inlineStr"/>
+      <c r="AP19" t="inlineStr"/>
+      <c r="AQ19" t="inlineStr"/>
+      <c r="AR19" t="inlineStr"/>
+      <c r="AS19" t="inlineStr"/>
+      <c r="AT19" t="inlineStr"/>
+      <c r="AU19" t="inlineStr"/>
+      <c r="AV19" t="inlineStr"/>
+      <c r="AW19" t="inlineStr"/>
+      <c r="AX19" t="inlineStr"/>
+      <c r="AY19" t="inlineStr"/>
+      <c r="AZ19" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
add and run XGB_007 latlon and XGB_008 chapinero filter - best spatial MAE so far
</commit_message>
<xml_diff>
--- a/02_outputs/model_registry.xlsx
+++ b/02_outputs/model_registry.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="registry" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="registry" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ19"/>
+  <dimension ref="A1:AZ21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2766,6 +2766,246 @@
       <c r="AY19" t="inlineStr"/>
       <c r="AZ19" t="inlineStr"/>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>XGB_007</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>31</v>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="n">
+        <v>5</v>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="n">
+        <v>0.17902</v>
+      </c>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>5x5</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>XGB_latlon_earlystop_XGB_007.csv</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>lat+lon como features geograficas directas. Early stopping=50 rondas. Mejor ronda=87. RandomizedSearch 50 iter. Sesgo Delta=+0.05153.</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="inlineStr"/>
+      <c r="X20" t="n">
+        <v>0.17922</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>0.00119</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>0.23075</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>0.00638</v>
+      </c>
+      <c r="AB20" t="inlineStr"/>
+      <c r="AC20" t="inlineStr"/>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>structural=7, osm=10, text=11, geo=2 (lat+lon), es_apartamento</t>
+        </is>
+      </c>
+      <c r="AE20" t="inlineStr"/>
+      <c r="AF20" t="inlineStr"/>
+      <c r="AG20" t="inlineStr"/>
+      <c r="AH20" t="inlineStr"/>
+      <c r="AI20" t="inlineStr"/>
+      <c r="AJ20" t="n">
+        <v>50</v>
+      </c>
+      <c r="AK20" t="inlineStr"/>
+      <c r="AL20" t="inlineStr"/>
+      <c r="AM20" t="n">
+        <v>87</v>
+      </c>
+      <c r="AN20" t="n">
+        <v>6</v>
+      </c>
+      <c r="AO20" t="inlineStr"/>
+      <c r="AP20" t="inlineStr"/>
+      <c r="AQ20" t="n">
+        <v>0.05153</v>
+      </c>
+      <c r="AR20" t="inlineStr"/>
+      <c r="AS20" t="n">
+        <v>0.0742</v>
+      </c>
+      <c r="AT20" t="n">
+        <v>0.614</v>
+      </c>
+      <c r="AU20" t="n">
+        <v>0.898</v>
+      </c>
+      <c r="AV20" t="n">
+        <v>2</v>
+      </c>
+      <c r="AW20" t="n">
+        <v>0.445</v>
+      </c>
+      <c r="AX20" t="n">
+        <v>3.1023</v>
+      </c>
+      <c r="AY20" t="n">
+        <v>0.094</v>
+      </c>
+      <c r="AZ20" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>XGB_008</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>31</v>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="n">
+        <v>5</v>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="n">
+        <v>0.17408</v>
+      </c>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>5x5</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>XGB_filtro_chapinero_earlystop_XGB_008.csv</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>Filtro train por rango IQR precio_m2 de Chapinero. Train: 38644 -&gt; 37918 obs. Rango: [-1,767,548, 12,489,100] COP/m2. Early stopping=50, mejor ronda=144. Sesgo Delta=+0.04783.</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="inlineStr"/>
+      <c r="X21" t="n">
+        <v>0.17798</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>0.00256</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>0.22582</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>0.01073</v>
+      </c>
+      <c r="AB21" t="inlineStr"/>
+      <c r="AC21" t="inlineStr"/>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>structural=7, osm=10, text=11, geo=2 (lat+lon), es_apartamento</t>
+        </is>
+      </c>
+      <c r="AE21" t="inlineStr"/>
+      <c r="AF21" t="inlineStr"/>
+      <c r="AG21" t="inlineStr"/>
+      <c r="AH21" t="inlineStr"/>
+      <c r="AI21" t="inlineStr"/>
+      <c r="AJ21" t="n">
+        <v>50</v>
+      </c>
+      <c r="AK21" t="inlineStr"/>
+      <c r="AL21" t="inlineStr"/>
+      <c r="AM21" t="n">
+        <v>144</v>
+      </c>
+      <c r="AN21" t="n">
+        <v>5</v>
+      </c>
+      <c r="AO21" t="inlineStr"/>
+      <c r="AP21" t="inlineStr"/>
+      <c r="AQ21" t="n">
+        <v>0.04783</v>
+      </c>
+      <c r="AR21" t="inlineStr"/>
+      <c r="AS21" t="n">
+        <v>0.07439999999999999</v>
+      </c>
+      <c r="AT21" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="AU21" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AV21" t="n">
+        <v>3</v>
+      </c>
+      <c r="AW21" t="n">
+        <v>0.3166</v>
+      </c>
+      <c r="AX21" t="n">
+        <v>4.537</v>
+      </c>
+      <c r="AY21" t="n">
+        <v>0.726</v>
+      </c>
+      <c r="AZ21" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
run XGB_009 KNN neighbors - best spatial MAE 0.211
</commit_message>
<xml_diff>
--- a/02_outputs/model_registry.xlsx
+++ b/02_outputs/model_registry.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ21"/>
+  <dimension ref="A1:BA22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -480,6 +480,7 @@
     <col width="12" customWidth="1" min="50" max="50"/>
     <col width="11" customWidth="1" min="51" max="51"/>
     <col width="15" customWidth="1" min="52" max="52"/>
+    <col width="11" customWidth="1" min="53" max="53"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -741,6 +742,11 @@
       <c r="AZ1" s="1" t="inlineStr">
         <is>
           <t>n_iter_search</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>k_vecinos</t>
         </is>
       </c>
     </row>
@@ -851,6 +857,7 @@
       <c r="AX2" t="inlineStr"/>
       <c r="AY2" t="inlineStr"/>
       <c r="AZ2" t="inlineStr"/>
+      <c r="BA2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -953,6 +960,7 @@
       <c r="AX3" t="inlineStr"/>
       <c r="AY3" t="inlineStr"/>
       <c r="AZ3" t="inlineStr"/>
+      <c r="BA3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1073,6 +1081,7 @@
       <c r="AX4" t="inlineStr"/>
       <c r="AY4" t="inlineStr"/>
       <c r="AZ4" t="inlineStr"/>
+      <c r="BA4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1183,6 +1192,7 @@
       <c r="AX5" t="inlineStr"/>
       <c r="AY5" t="inlineStr"/>
       <c r="AZ5" t="inlineStr"/>
+      <c r="BA5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1293,6 +1303,7 @@
       <c r="AX6" t="inlineStr"/>
       <c r="AY6" t="inlineStr"/>
       <c r="AZ6" t="inlineStr"/>
+      <c r="BA6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1405,6 +1416,7 @@
       <c r="AX7" t="inlineStr"/>
       <c r="AY7" t="inlineStr"/>
       <c r="AZ7" t="inlineStr"/>
+      <c r="BA7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1517,6 +1529,7 @@
       <c r="AX8" t="inlineStr"/>
       <c r="AY8" t="inlineStr"/>
       <c r="AZ8" t="inlineStr"/>
+      <c r="BA8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1629,6 +1642,7 @@
       <c r="AX9" t="inlineStr"/>
       <c r="AY9" t="inlineStr"/>
       <c r="AZ9" t="inlineStr"/>
+      <c r="BA9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1735,6 +1749,7 @@
       <c r="AX10" t="inlineStr"/>
       <c r="AY10" t="inlineStr"/>
       <c r="AZ10" t="inlineStr"/>
+      <c r="BA10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1843,6 +1858,7 @@
       <c r="AX11" t="inlineStr"/>
       <c r="AY11" t="inlineStr"/>
       <c r="AZ11" t="inlineStr"/>
+      <c r="BA11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1955,6 +1971,7 @@
       <c r="AX12" t="inlineStr"/>
       <c r="AY12" t="inlineStr"/>
       <c r="AZ12" t="inlineStr"/>
+      <c r="BA12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2067,6 +2084,7 @@
       <c r="AX13" t="inlineStr"/>
       <c r="AY13" t="inlineStr"/>
       <c r="AZ13" t="inlineStr"/>
+      <c r="BA13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2179,6 +2197,7 @@
       <c r="AX14" t="inlineStr"/>
       <c r="AY14" t="inlineStr"/>
       <c r="AZ14" t="inlineStr"/>
+      <c r="BA14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2301,6 +2320,7 @@
       <c r="AZ15" t="n">
         <v>50</v>
       </c>
+      <c r="BA15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2419,6 +2439,7 @@
       <c r="AZ16" t="n">
         <v>50</v>
       </c>
+      <c r="BA16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2537,6 +2558,7 @@
       <c r="AZ17" t="n">
         <v>150</v>
       </c>
+      <c r="BA17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2645,6 +2667,7 @@
       <c r="AX18" t="inlineStr"/>
       <c r="AY18" t="inlineStr"/>
       <c r="AZ18" t="inlineStr"/>
+      <c r="BA18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2765,6 +2788,7 @@
       <c r="AX19" t="inlineStr"/>
       <c r="AY19" t="inlineStr"/>
       <c r="AZ19" t="inlineStr"/>
+      <c r="BA19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2885,6 +2909,7 @@
       <c r="AZ20" t="n">
         <v>50</v>
       </c>
+      <c r="BA20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3005,6 +3030,130 @@
       <c r="AZ21" t="n">
         <v>50</v>
       </c>
+      <c r="BA21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>XGB_009</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>32</v>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="n">
+        <v>5</v>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="n">
+        <v>0.16854</v>
+      </c>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>5x5</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>XGB_knn30_latlon_earlystop_XGB_009.csv</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>Base XGB_007 + precio mediano K=30 vecinos (haversine, LOO). Early stopping espacial bloque mas grande. Sesgo Delta=+0.03480.</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr"/>
+      <c r="W22" t="inlineStr"/>
+      <c r="X22" t="n">
+        <v>0.17598</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>0.0016</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>0.21079</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>0.00991</v>
+      </c>
+      <c r="AB22" t="inlineStr"/>
+      <c r="AC22" t="inlineStr"/>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>structural=7, osm=10, text=11, geo=2 (lat+lon), precio_vecinos=1 (K=30 LOO), es_apartamento</t>
+        </is>
+      </c>
+      <c r="AE22" t="inlineStr"/>
+      <c r="AF22" t="inlineStr"/>
+      <c r="AG22" t="inlineStr"/>
+      <c r="AH22" t="inlineStr"/>
+      <c r="AI22" t="inlineStr"/>
+      <c r="AJ22" t="n">
+        <v>50</v>
+      </c>
+      <c r="AK22" t="inlineStr"/>
+      <c r="AL22" t="inlineStr"/>
+      <c r="AM22" t="n">
+        <v>265</v>
+      </c>
+      <c r="AN22" t="n">
+        <v>6</v>
+      </c>
+      <c r="AO22" t="inlineStr"/>
+      <c r="AP22" t="inlineStr"/>
+      <c r="AQ22" t="n">
+        <v>0.0348</v>
+      </c>
+      <c r="AR22" t="inlineStr"/>
+      <c r="AS22" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="AT22" t="n">
+        <v>0.749</v>
+      </c>
+      <c r="AU22" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="AV22" t="n">
+        <v>6</v>
+      </c>
+      <c r="AW22" t="n">
+        <v>0.321</v>
+      </c>
+      <c r="AX22" t="n">
+        <v>3.1131</v>
+      </c>
+      <c r="AY22" t="n">
+        <v>0.669</v>
+      </c>
+      <c r="AZ22" t="n">
+        <v>50</v>
+      </c>
+      <c r="BA22" t="n">
+        <v>30</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
remove XGB_010 ensemble - not a valid algorithm for PS3
</commit_message>
<xml_diff>
--- a/02_outputs/model_registry.xlsx
+++ b/02_outputs/model_registry.xlsx
@@ -425,14 +425,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA22"/>
+  <dimension ref="A1:BA23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
@@ -3155,6 +3155,85 @@
         <v>30</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>XGB_010</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Ensemble</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>XGB_007 + XGB_009</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>XGB_ensemble_007_009_XGB_010.csv</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>Ensemble simple: promedio ponderado XGB_007 (w=0.5) y XGB_009 (w=0.5). XGB_007 MAE Kaggle=225M, XGB_009 MAE Kaggle=207M. Promedio en escala COP para minimizar MAE directamente.</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr"/>
+      <c r="W23" t="inlineStr"/>
+      <c r="X23" t="inlineStr"/>
+      <c r="Y23" t="inlineStr"/>
+      <c r="Z23" t="inlineStr"/>
+      <c r="AA23" t="inlineStr"/>
+      <c r="AB23" t="inlineStr"/>
+      <c r="AC23" t="inlineStr"/>
+      <c r="AD23" t="inlineStr"/>
+      <c r="AE23" t="inlineStr"/>
+      <c r="AF23" t="inlineStr"/>
+      <c r="AG23" t="inlineStr"/>
+      <c r="AH23" t="inlineStr"/>
+      <c r="AI23" t="inlineStr"/>
+      <c r="AJ23" t="inlineStr"/>
+      <c r="AK23" t="inlineStr"/>
+      <c r="AL23" t="inlineStr"/>
+      <c r="AM23" t="inlineStr"/>
+      <c r="AN23" t="inlineStr"/>
+      <c r="AO23" t="inlineStr"/>
+      <c r="AP23" t="inlineStr"/>
+      <c r="AQ23" t="inlineStr"/>
+      <c r="AR23" t="inlineStr"/>
+      <c r="AS23" t="inlineStr"/>
+      <c r="AT23" t="inlineStr"/>
+      <c r="AU23" t="inlineStr"/>
+      <c r="AV23" t="inlineStr"/>
+      <c r="AW23" t="inlineStr"/>
+      <c r="AX23" t="inlineStr"/>
+      <c r="AY23" t="inlineStr"/>
+      <c r="AZ23" t="inlineStr"/>
+      <c r="BA23" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: run XGB_010 KNN weighted - best spatial MAE 0.173
</commit_message>
<xml_diff>
--- a/02_outputs/model_registry.xlsx
+++ b/02_outputs/model_registry.xlsx
@@ -432,7 +432,7 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
@@ -3169,70 +3169,114 @@
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Ensemble</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>XGB_007 + XGB_009</t>
-        </is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>32</v>
       </c>
       <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
+      <c r="G23" t="n">
+        <v>5</v>
+      </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
+      <c r="M23" t="n">
+        <v>0.13865</v>
+      </c>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>5x5</t>
+        </is>
+      </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>XGB_ensemble_007_009_XGB_010.csv</t>
+          <t>XGB_knn30_weighted_earlystop_XGB_010.csv</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>Ensemble simple: promedio ponderado XGB_007 (w=0.5) y XGB_009 (w=0.5). XGB_007 MAE Kaggle=225M, XGB_009 MAE Kaggle=207M. Promedio en escala COP para minimizar MAE directamente.</t>
+          <t>Base XGB_009 + precio ponderado por distancia K=30 vecinos. peso_i=1/dist_i (haversine km). LOO en train. Early stopping espacial. Sesgo Delta=+0.02231.</t>
         </is>
       </c>
       <c r="V23" t="inlineStr"/>
       <c r="W23" t="inlineStr"/>
-      <c r="X23" t="inlineStr"/>
-      <c r="Y23" t="inlineStr"/>
-      <c r="Z23" t="inlineStr"/>
-      <c r="AA23" t="inlineStr"/>
+      <c r="X23" t="n">
+        <v>0.15029</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>0.00154</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>0.1726</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>0.00742</v>
+      </c>
       <c r="AB23" t="inlineStr"/>
       <c r="AC23" t="inlineStr"/>
-      <c r="AD23" t="inlineStr"/>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>structural=7, osm=10, text=11, geo=2 (lat+lon), precio_vecinos_ponderado=1 (K=30 LOO haversine), es_apartamento</t>
+        </is>
+      </c>
       <c r="AE23" t="inlineStr"/>
       <c r="AF23" t="inlineStr"/>
       <c r="AG23" t="inlineStr"/>
       <c r="AH23" t="inlineStr"/>
       <c r="AI23" t="inlineStr"/>
-      <c r="AJ23" t="inlineStr"/>
+      <c r="AJ23" t="n">
+        <v>50</v>
+      </c>
       <c r="AK23" t="inlineStr"/>
       <c r="AL23" t="inlineStr"/>
-      <c r="AM23" t="inlineStr"/>
-      <c r="AN23" t="inlineStr"/>
+      <c r="AM23" t="n">
+        <v>141</v>
+      </c>
+      <c r="AN23" t="n">
+        <v>8</v>
+      </c>
       <c r="AO23" t="inlineStr"/>
       <c r="AP23" t="inlineStr"/>
-      <c r="AQ23" t="inlineStr"/>
+      <c r="AQ23" t="n">
+        <v>0.02231</v>
+      </c>
       <c r="AR23" t="inlineStr"/>
-      <c r="AS23" t="inlineStr"/>
-      <c r="AT23" t="inlineStr"/>
-      <c r="AU23" t="inlineStr"/>
-      <c r="AV23" t="inlineStr"/>
-      <c r="AW23" t="inlineStr"/>
-      <c r="AX23" t="inlineStr"/>
-      <c r="AY23" t="inlineStr"/>
-      <c r="AZ23" t="inlineStr"/>
-      <c r="BA23" t="inlineStr"/>
+      <c r="AS23" t="n">
+        <v>0.0639</v>
+      </c>
+      <c r="AT23" t="n">
+        <v>0.998</v>
+      </c>
+      <c r="AU23" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="AV23" t="n">
+        <v>2</v>
+      </c>
+      <c r="AW23" t="n">
+        <v>0.4868</v>
+      </c>
+      <c r="AX23" t="n">
+        <v>2.5179</v>
+      </c>
+      <c r="AY23" t="n">
+        <v>0.4856</v>
+      </c>
+      <c r="AZ23" t="n">
+        <v>50</v>
+      </c>
+      <c r="BA23" t="n">
+        <v>30</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: add XGB_009 and XGB_010 to registry
</commit_message>
<xml_diff>
--- a/02_outputs/model_registry.xlsx
+++ b/02_outputs/model_registry.xlsx
@@ -3040,7 +3040,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -3163,7 +3163,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>

</xml_diff>

<commit_message>
fix: update model registry with new binary data
</commit_message>
<xml_diff>
--- a/02_outputs/model_registry.xlsx
+++ b/02_outputs/model_registry.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbook/Documents/Documentos/MeCA/202601/BDML/Problem_sets/Problem-Set-3-Making-Money-with-ML/02_outputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5AE63BB-2A81-2946-9869-33CE3DB01CD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE109E11-A5F0-DE49-A1F1-1CBD63680F32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20" yWindow="660" windowWidth="29400" windowHeight="17260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="registry" sheetId="1" r:id="rId1"/>
@@ -869,6 +869,8 @@
   <dimension ref="A1:BG24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="3" max="3" width="20.6640625" customWidth="1"/>
+    <col min="4" max="4" width="23.1640625" customWidth="1"/>
     <col min="14" max="14" width="10.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2166,6 +2168,9 @@
       <c r="M19">
         <v>0.13739000000000001</v>
       </c>
+      <c r="N19">
+        <v>216987903.08000001</v>
+      </c>
       <c r="S19" t="s">
         <v>63</v>
       </c>
@@ -2547,6 +2552,9 @@
       </c>
       <c r="M24">
         <v>0.14644199999999999</v>
+      </c>
+      <c r="N24">
+        <v>199851631.65000001</v>
       </c>
       <c r="T24" t="s">
         <v>158</v>

</xml_diff>

<commit_message>
outputs: pipeline completo LR_001 EN_002 CART_002 RF_005 XGB_009 NN_003 SL_003
</commit_message>
<xml_diff>
--- a/02_outputs/model_registry.xlsx
+++ b/02_outputs/model_registry.xlsx
@@ -1507,7 +1507,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>RF_005</t>
+          <t>CART_001</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1517,16 +1517,16 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Equipo</t>
+          <t>Dani</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>CART</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
@@ -1538,7 +1538,7 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
-        <v>0.16414</v>
+        <v>0.19418</v>
       </c>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
@@ -1552,33 +1552,33 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>RF_ntrees500_d15_leaf5_mfsqrt_cv5_gridESP_RF_005.csv</t>
+          <t>CART_dNone_leaf1_ccp00_cv5_CART_001.csv</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>Grid search max_depth=[8, 10, 15] via CV espacial. Best depth=15. n_estimators=500, min_samples_leaf=5. Features completas. Sesgo Δ=+0.07192.</t>
+          <t>Baseline: solo features estructurales + es_apartamento. Defaults sklearn: depth=None, leaf=1, ccp=0. Sin OSM ni texto. Sesgo Δ=+0.03824.</t>
         </is>
       </c>
       <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr"/>
       <c r="X8" t="n">
-        <v>0.19172</v>
+        <v>0.26502</v>
       </c>
       <c r="Y8" t="n">
-        <v>0.00195</v>
+        <v>0.00274</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.26364</v>
+        <v>0.30326</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.00848</v>
+        <v>0.011</v>
       </c>
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>structural=7, text=11, osm=10, es_apartamento</t>
+          <t>structural=7, text=0, osm=0, es_apartamento</t>
         </is>
       </c>
       <c r="AE8" t="inlineStr"/>
@@ -1589,24 +1589,18 @@
       <c r="AJ8" t="inlineStr"/>
       <c r="AK8" t="inlineStr"/>
       <c r="AL8" t="inlineStr"/>
-      <c r="AM8" t="n">
-        <v>500</v>
-      </c>
-      <c r="AN8" t="n">
-        <v>15</v>
-      </c>
+      <c r="AM8" t="inlineStr"/>
+      <c r="AN8" t="inlineStr"/>
       <c r="AO8" t="n">
-        <v>5</v>
-      </c>
-      <c r="AP8" t="inlineStr">
-        <is>
-          <t>sqrt</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="AP8" t="inlineStr"/>
       <c r="AQ8" t="n">
-        <v>0.07192</v>
-      </c>
-      <c r="AR8" t="inlineStr"/>
+        <v>0.03824</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>0</v>
+      </c>
       <c r="AS8" t="inlineStr"/>
       <c r="AT8" t="inlineStr"/>
       <c r="AU8" t="inlineStr"/>
@@ -1626,7 +1620,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CART_001</t>
+          <t>XGB_001</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1641,7 +1635,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -1657,7 +1651,7 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
-        <v>0.19418</v>
+        <v>0.23932</v>
       </c>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
@@ -1671,27 +1665,27 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>CART_dNone_leaf1_ccp00_cv5_CART_001.csv</t>
+          <t>XGB_nest100_d6_lr03_cv5_XGB_001.csv</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>Baseline: solo features estructurales + es_apartamento. Defaults sklearn: depth=None, leaf=1, ccp=0. Sin OSM ni texto. Sesgo Δ=+0.03824.</t>
+          <t>Baseline: solo estructurales + es_apartamento. Defaults XGBoost: n_est=100, depth=6, lr=0.3. Sin OSM ni texto. Sesgo Delta=+0.02424.</t>
         </is>
       </c>
       <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr"/>
       <c r="X9" t="n">
-        <v>0.26502</v>
+        <v>0.25235</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.00274</v>
+        <v>0.00246</v>
       </c>
       <c r="Z9" t="n">
-        <v>0.30326</v>
+        <v>0.27659</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.011</v>
+        <v>0.01182</v>
       </c>
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr"/>
@@ -1708,21 +1702,27 @@
       <c r="AJ9" t="inlineStr"/>
       <c r="AK9" t="inlineStr"/>
       <c r="AL9" t="inlineStr"/>
-      <c r="AM9" t="inlineStr"/>
-      <c r="AN9" t="inlineStr"/>
-      <c r="AO9" t="n">
-        <v>1</v>
-      </c>
+      <c r="AM9" t="n">
+        <v>100</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>6</v>
+      </c>
+      <c r="AO9" t="inlineStr"/>
       <c r="AP9" t="inlineStr"/>
       <c r="AQ9" t="n">
-        <v>0.03824</v>
-      </c>
-      <c r="AR9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS9" t="inlineStr"/>
-      <c r="AT9" t="inlineStr"/>
-      <c r="AU9" t="inlineStr"/>
+        <v>0.02424</v>
+      </c>
+      <c r="AR9" t="inlineStr"/>
+      <c r="AS9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AT9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>1</v>
+      </c>
       <c r="AV9" t="inlineStr"/>
       <c r="AW9" t="inlineStr"/>
       <c r="AX9" t="inlineStr"/>
@@ -1739,7 +1739,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CART_002</t>
+          <t>XGB_002</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1754,7 +1754,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -1770,7 +1770,7 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
-        <v>0.22825</v>
+        <v>0.1391</v>
       </c>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
@@ -1784,27 +1784,27 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>CART_d10_leaf20_ccp00001_cv5_CART_002.csv</t>
+          <t>XGB_nest100_d6_lr03_allfeats_cv5_XGB_002.csv</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>All features: estructurales + OSM + texto. GridSearchCV espacial. Params: {'ccp_alpha': 0.0001, 'max_depth': 10, 'min_samples_leaf': 20}. Sesgo Delta=+0.04144.</t>
+          <t>All features: estructurales + OSM + texto. Defaults XGBoost sin tuning. Sesgo Delta=+0.10189.</t>
         </is>
       </c>
       <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr"/>
       <c r="X10" t="n">
-        <v>0.2326</v>
+        <v>0.1737</v>
       </c>
       <c r="Y10" t="n">
-        <v>0.00216</v>
+        <v>0.00133</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.27405</v>
+        <v>0.2756</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.01087</v>
+        <v>0.01177</v>
       </c>
       <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr"/>
@@ -1821,23 +1821,27 @@
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr"/>
       <c r="AL10" t="inlineStr"/>
-      <c r="AM10" t="inlineStr"/>
+      <c r="AM10" t="n">
+        <v>100</v>
+      </c>
       <c r="AN10" t="n">
-        <v>10</v>
-      </c>
-      <c r="AO10" t="n">
-        <v>20</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="AO10" t="inlineStr"/>
       <c r="AP10" t="inlineStr"/>
       <c r="AQ10" t="n">
-        <v>0.04144</v>
-      </c>
-      <c r="AR10" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="AS10" t="inlineStr"/>
-      <c r="AT10" t="inlineStr"/>
-      <c r="AU10" t="inlineStr"/>
+        <v>0.10189</v>
+      </c>
+      <c r="AR10" t="inlineStr"/>
+      <c r="AS10" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>1</v>
+      </c>
       <c r="AV10" t="inlineStr"/>
       <c r="AW10" t="inlineStr"/>
       <c r="AX10" t="inlineStr"/>
@@ -1854,7 +1858,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>XGB_001</t>
+          <t>XGB_003</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1873,7 +1877,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
@@ -1885,7 +1889,7 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
-        <v>0.23932</v>
+        <v>0.14165</v>
       </c>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
@@ -1899,33 +1903,33 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>XGB_nest100_d6_lr03_cv5_XGB_001.csv</t>
+          <t>XGB_nest300_d7_lr005_cv5_XGB_003.csv</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>Baseline: solo estructurales + es_apartamento. Defaults XGBoost: n_est=100, depth=6, lr=0.3. Sin OSM ni texto. Sesgo Delta=+0.02424.</t>
+          <t>Depth tuning: GridSearch sobre max_depth y learning_rate. n_estimators fijo=300. Params: {'learning_rate': 0.05, 'max_depth': 7}. Sesgo Delta=+0.08760.</t>
         </is>
       </c>
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
       <c r="X11" t="n">
-        <v>0.25235</v>
+        <v>0.17131</v>
       </c>
       <c r="Y11" t="n">
-        <v>0.00246</v>
+        <v>0.00134</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.27659</v>
+        <v>0.25891</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.01182</v>
+        <v>0.00825</v>
       </c>
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>
       <c r="AD11" t="inlineStr">
         <is>
-          <t>structural=7, text=0, osm=0, es_apartamento</t>
+          <t>structural=7, osm=10, text=11, es_apartamento</t>
         </is>
       </c>
       <c r="AE11" t="inlineStr"/>
@@ -1937,25 +1941,25 @@
       <c r="AK11" t="inlineStr"/>
       <c r="AL11" t="inlineStr"/>
       <c r="AM11" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="AN11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AO11" t="inlineStr"/>
       <c r="AP11" t="inlineStr"/>
       <c r="AQ11" t="n">
-        <v>0.02424</v>
+        <v>0.0876</v>
       </c>
       <c r="AR11" t="inlineStr"/>
       <c r="AS11" t="n">
-        <v>0.3</v>
+        <v>0.05</v>
       </c>
       <c r="AT11" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="AU11" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="AV11" t="inlineStr"/>
       <c r="AW11" t="inlineStr"/>
@@ -1973,7 +1977,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>XGB_002</t>
+          <t>XGB_004</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2004,7 +2008,7 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
-        <v>0.1391</v>
+        <v>0.18526</v>
       </c>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
@@ -2018,27 +2022,27 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>XGB_nest100_d6_lr03_allfeats_cv5_XGB_002.csv</t>
+          <t>XGB_nest356_d6_lr0078_cv5_XGB_004.csv</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>All features: estructurales + OSM + texto. Defaults XGBoost sin tuning. Sesgo Delta=+0.10189.</t>
+          <t>Tuning exhaustivo: RandomizedSearchCV 50 iter, 9 hiperparametros, CV espacial. Params: {'colsample_bytree': 0.6356745158869479, 'gamma': 0.41436875457596467, 'learning_rate': 0.07778313207178196, 'max_depth': 6, 'min_child_weight': 9, 'n_estimators': 356, 'reg_alpha': 0.8021969807540397, 'reg_lambda': 0.8354778965589686, 'subsample': 0.9947547746402069}. Sesgo Delta=+0.06037.</t>
         </is>
       </c>
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr"/>
       <c r="X12" t="n">
-        <v>0.1737</v>
+        <v>0.19596</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.00133</v>
+        <v>0.0019</v>
       </c>
       <c r="Z12" t="n">
-        <v>0.2756</v>
+        <v>0.25634</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.01177</v>
+        <v>0.00665</v>
       </c>
       <c r="AB12" t="inlineStr"/>
       <c r="AC12" t="inlineStr"/>
@@ -2056,7 +2060,7 @@
       <c r="AK12" t="inlineStr"/>
       <c r="AL12" t="inlineStr"/>
       <c r="AM12" t="n">
-        <v>100</v>
+        <v>356</v>
       </c>
       <c r="AN12" t="n">
         <v>6</v>
@@ -2064,23 +2068,33 @@
       <c r="AO12" t="inlineStr"/>
       <c r="AP12" t="inlineStr"/>
       <c r="AQ12" t="n">
-        <v>0.10189</v>
+        <v>0.06037</v>
       </c>
       <c r="AR12" t="inlineStr"/>
       <c r="AS12" t="n">
-        <v>0.3</v>
+        <v>0.07779999999999999</v>
       </c>
       <c r="AT12" t="n">
-        <v>1</v>
+        <v>0.995</v>
       </c>
       <c r="AU12" t="n">
-        <v>1</v>
-      </c>
-      <c r="AV12" t="inlineStr"/>
-      <c r="AW12" t="inlineStr"/>
-      <c r="AX12" t="inlineStr"/>
-      <c r="AY12" t="inlineStr"/>
-      <c r="AZ12" t="inlineStr"/>
+        <v>0.636</v>
+      </c>
+      <c r="AV12" t="n">
+        <v>9</v>
+      </c>
+      <c r="AW12" t="n">
+        <v>0.4144</v>
+      </c>
+      <c r="AX12" t="n">
+        <v>0.8355</v>
+      </c>
+      <c r="AY12" t="n">
+        <v>0.8022</v>
+      </c>
+      <c r="AZ12" t="n">
+        <v>50</v>
+      </c>
       <c r="BA12" t="inlineStr"/>
       <c r="BB12" t="inlineStr"/>
       <c r="BC12" t="inlineStr"/>
@@ -2092,7 +2106,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>XGB_003</t>
+          <t>XGB_005</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2100,18 +2114,14 @@
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Dani</t>
-        </is>
-      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
@@ -2123,7 +2133,7 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
-        <v>0.14165</v>
+        <v>0.14478</v>
       </c>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
@@ -2137,33 +2147,33 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>XGB_nest300_d7_lr005_cv5_XGB_003.csv</t>
+          <t>XGB_spatial_nest304_d4_lr0014_cv5_XGB_005.csv</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>Depth tuning: GridSearch sobre max_depth y learning_rate. n_estimators fijo=300. Params: {'learning_rate': 0.05, 'max_depth': 7}. Sesgo Delta=+0.08760.</t>
+          <t>All features + target encoding espacial leave-one-out. RandomizedSearchCV 50 iter, CV espacial. Params: {'colsample_bytree': 0.6594878151468806, 'gamma': 0.4224376554847273, 'learning_rate': 0.014421667789806915, 'max_depth': 4, 'min_child_weight': 3, 'n_estimators': 304, 'reg_alpha': 0.4960374542934062, 'reg_lambda': 3.6180066141137273, 'subsample': 0.739334641781279}. Sesgo Delta=+0.14700.</t>
         </is>
       </c>
       <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr"/>
       <c r="X13" t="n">
-        <v>0.17131</v>
+        <v>0.14821</v>
       </c>
       <c r="Y13" t="n">
-        <v>0.00134</v>
+        <v>0.00297</v>
       </c>
       <c r="Z13" t="n">
-        <v>0.25891</v>
+        <v>0.29521</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.00825</v>
+        <v>0.02317</v>
       </c>
       <c r="AB13" t="inlineStr"/>
       <c r="AC13" t="inlineStr"/>
       <c r="AD13" t="inlineStr">
         <is>
-          <t>structural=7, osm=10, text=11, es_apartamento</t>
+          <t>structural=7, osm=10, text=11, target_espacial=1, es_apartamento</t>
         </is>
       </c>
       <c r="AE13" t="inlineStr"/>
@@ -2175,31 +2185,41 @@
       <c r="AK13" t="inlineStr"/>
       <c r="AL13" t="inlineStr"/>
       <c r="AM13" t="n">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="AN13" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="AO13" t="inlineStr"/>
       <c r="AP13" t="inlineStr"/>
       <c r="AQ13" t="n">
-        <v>0.0876</v>
+        <v>0.147</v>
       </c>
       <c r="AR13" t="inlineStr"/>
       <c r="AS13" t="n">
-        <v>0.05</v>
+        <v>0.0144</v>
       </c>
       <c r="AT13" t="n">
-        <v>0.8</v>
+        <v>0.739</v>
       </c>
       <c r="AU13" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AV13" t="inlineStr"/>
-      <c r="AW13" t="inlineStr"/>
-      <c r="AX13" t="inlineStr"/>
-      <c r="AY13" t="inlineStr"/>
-      <c r="AZ13" t="inlineStr"/>
+        <v>0.659</v>
+      </c>
+      <c r="AV13" t="n">
+        <v>3</v>
+      </c>
+      <c r="AW13" t="n">
+        <v>0.4224</v>
+      </c>
+      <c r="AX13" t="n">
+        <v>3.618</v>
+      </c>
+      <c r="AY13" t="n">
+        <v>0.496</v>
+      </c>
+      <c r="AZ13" t="n">
+        <v>50</v>
+      </c>
       <c r="BA13" t="inlineStr"/>
       <c r="BB13" t="inlineStr"/>
       <c r="BC13" t="inlineStr"/>
@@ -2211,7 +2231,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>XGB_004</t>
+          <t>XGB_006</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2219,11 +2239,7 @@
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Dani</t>
-        </is>
-      </c>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
           <t>XGBoost</t>
@@ -2242,7 +2258,7 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
-        <v>0.18526</v>
+        <v>0.16684</v>
       </c>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
@@ -2256,27 +2272,27 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>XGB_nest356_d6_lr0078_cv5_XGB_004.csv</t>
+          <t>XGB_iter150_nest564_d8_lr0075_cv5_XGB_006.csv</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>Tuning exhaustivo: RandomizedSearchCV 50 iter, 9 hiperparametros, CV espacial. Params: {'colsample_bytree': 0.6356745158869479, 'gamma': 0.41436875457596467, 'learning_rate': 0.07778313207178196, 'max_depth': 6, 'min_child_weight': 9, 'n_estimators': 356, 'reg_alpha': 0.8021969807540397, 'reg_lambda': 0.8354778965589686, 'subsample': 0.9947547746402069}. Sesgo Delta=+0.06037.</t>
+          <t>All features. RandomizedSearchCV 150 iter (3x XGB_004). Mismo espacio de busqueda que XGB_004 para comparacion justa. Params: {'colsample_bytree': 0.8812293428703453, 'gamma': 0.43838281838087473, 'learning_rate': 0.07499553225602242, 'max_depth': 8, 'min_child_weight': 4, 'n_estimators': 564, 'reg_alpha': 0.12748866233198242, 'reg_lambda': 2.2877928075216527, 'subsample': 0.9189181463118214}. Sesgo Delta=+0.06906.</t>
         </is>
       </c>
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr"/>
       <c r="X14" t="n">
-        <v>0.19596</v>
+        <v>0.18619</v>
       </c>
       <c r="Y14" t="n">
-        <v>0.0019</v>
+        <v>0.00112</v>
       </c>
       <c r="Z14" t="n">
-        <v>0.25634</v>
+        <v>0.25525</v>
       </c>
       <c r="AA14" t="n">
-        <v>0.00665</v>
+        <v>0.00721</v>
       </c>
       <c r="AB14" t="inlineStr"/>
       <c r="AC14" t="inlineStr"/>
@@ -2294,40 +2310,40 @@
       <c r="AK14" t="inlineStr"/>
       <c r="AL14" t="inlineStr"/>
       <c r="AM14" t="n">
-        <v>356</v>
+        <v>564</v>
       </c>
       <c r="AN14" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AO14" t="inlineStr"/>
       <c r="AP14" t="inlineStr"/>
       <c r="AQ14" t="n">
-        <v>0.06037</v>
+        <v>0.06906</v>
       </c>
       <c r="AR14" t="inlineStr"/>
       <c r="AS14" t="n">
-        <v>0.07779999999999999</v>
+        <v>0.075</v>
       </c>
       <c r="AT14" t="n">
-        <v>0.995</v>
+        <v>0.919</v>
       </c>
       <c r="AU14" t="n">
-        <v>0.636</v>
+        <v>0.881</v>
       </c>
       <c r="AV14" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="AW14" t="n">
-        <v>0.4144</v>
+        <v>0.4384</v>
       </c>
       <c r="AX14" t="n">
-        <v>0.8355</v>
+        <v>2.2878</v>
       </c>
       <c r="AY14" t="n">
-        <v>0.8022</v>
+        <v>0.1275</v>
       </c>
       <c r="AZ14" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="BA14" t="inlineStr"/>
       <c r="BB14" t="inlineStr"/>
@@ -2340,12 +2356,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>XGB_005</t>
+          <t>XGB_007</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
@@ -2355,7 +2371,7 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
@@ -2367,7 +2383,7 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
-        <v>0.14478</v>
+        <v>0.17902</v>
       </c>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
@@ -2381,33 +2397,33 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>XGB_spatial_nest304_d4_lr0014_cv5_XGB_005.csv</t>
+          <t>XGB_latlon_earlystop_XGB_007.csv</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>All features + target encoding espacial leave-one-out. RandomizedSearchCV 50 iter, CV espacial. Params: {'colsample_bytree': 0.6594878151468806, 'gamma': 0.4224376554847273, 'learning_rate': 0.014421667789806915, 'max_depth': 4, 'min_child_weight': 3, 'n_estimators': 304, 'reg_alpha': 0.4960374542934062, 'reg_lambda': 3.6180066141137273, 'subsample': 0.739334641781279}. Sesgo Delta=+0.14700.</t>
+          <t>lat+lon como features geograficas directas. Early stopping=50 rondas. Mejor ronda=87. RandomizedSearch 50 iter. Sesgo Delta=+0.05153.</t>
         </is>
       </c>
       <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr"/>
       <c r="X15" t="n">
-        <v>0.14821</v>
+        <v>0.17922</v>
       </c>
       <c r="Y15" t="n">
-        <v>0.00297</v>
+        <v>0.00119</v>
       </c>
       <c r="Z15" t="n">
-        <v>0.29521</v>
+        <v>0.23075</v>
       </c>
       <c r="AA15" t="n">
-        <v>0.02317</v>
+        <v>0.00638</v>
       </c>
       <c r="AB15" t="inlineStr"/>
       <c r="AC15" t="inlineStr"/>
       <c r="AD15" t="inlineStr">
         <is>
-          <t>structural=7, osm=10, text=11, target_espacial=1, es_apartamento</t>
+          <t>structural=7, osm=10, text=11, geo=2 (lat+lon), es_apartamento</t>
         </is>
       </c>
       <c r="AE15" t="inlineStr"/>
@@ -2415,41 +2431,43 @@
       <c r="AG15" t="inlineStr"/>
       <c r="AH15" t="inlineStr"/>
       <c r="AI15" t="inlineStr"/>
-      <c r="AJ15" t="inlineStr"/>
+      <c r="AJ15" t="n">
+        <v>50</v>
+      </c>
       <c r="AK15" t="inlineStr"/>
       <c r="AL15" t="inlineStr"/>
       <c r="AM15" t="n">
-        <v>304</v>
+        <v>87</v>
       </c>
       <c r="AN15" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AO15" t="inlineStr"/>
       <c r="AP15" t="inlineStr"/>
       <c r="AQ15" t="n">
-        <v>0.147</v>
+        <v>0.05153</v>
       </c>
       <c r="AR15" t="inlineStr"/>
       <c r="AS15" t="n">
-        <v>0.0144</v>
+        <v>0.0742</v>
       </c>
       <c r="AT15" t="n">
-        <v>0.739</v>
+        <v>0.614</v>
       </c>
       <c r="AU15" t="n">
-        <v>0.659</v>
+        <v>0.898</v>
       </c>
       <c r="AV15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AW15" t="n">
-        <v>0.4224</v>
+        <v>0.445</v>
       </c>
       <c r="AX15" t="n">
-        <v>3.618</v>
+        <v>3.1023</v>
       </c>
       <c r="AY15" t="n">
-        <v>0.496</v>
+        <v>0.094</v>
       </c>
       <c r="AZ15" t="n">
         <v>50</v>
@@ -2465,12 +2483,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>XGB_006</t>
+          <t>XGB_008</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -2480,7 +2498,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="n">
@@ -2492,7 +2510,7 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
-        <v>0.16684</v>
+        <v>0.17408</v>
       </c>
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
@@ -2506,33 +2524,33 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>XGB_iter150_nest564_d8_lr0075_cv5_XGB_006.csv</t>
+          <t>XGB_filtro_chapinero_earlystop_XGB_008.csv</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>All features. RandomizedSearchCV 150 iter (3x XGB_004). Mismo espacio de busqueda que XGB_004 para comparacion justa. Params: {'colsample_bytree': 0.8812293428703453, 'gamma': 0.43838281838087473, 'learning_rate': 0.07499553225602242, 'max_depth': 8, 'min_child_weight': 4, 'n_estimators': 564, 'reg_alpha': 0.12748866233198242, 'reg_lambda': 2.2877928075216527, 'subsample': 0.9189181463118214}. Sesgo Delta=+0.06906.</t>
+          <t>Filtro train por rango IQR precio_m2 de Chapinero. Train: 38644 -&gt; 37918 obs. Rango: [-1,767,548, 12,489,100] COP/m2. Early stopping=50, mejor ronda=144. Sesgo Delta=+0.04783.</t>
         </is>
       </c>
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr"/>
       <c r="X16" t="n">
-        <v>0.18619</v>
+        <v>0.17798</v>
       </c>
       <c r="Y16" t="n">
-        <v>0.00112</v>
+        <v>0.00256</v>
       </c>
       <c r="Z16" t="n">
-        <v>0.25525</v>
+        <v>0.22582</v>
       </c>
       <c r="AA16" t="n">
-        <v>0.00721</v>
+        <v>0.01073</v>
       </c>
       <c r="AB16" t="inlineStr"/>
       <c r="AC16" t="inlineStr"/>
       <c r="AD16" t="inlineStr">
         <is>
-          <t>structural=7, osm=10, text=11, es_apartamento</t>
+          <t>structural=7, osm=10, text=11, geo=2 (lat+lon), es_apartamento</t>
         </is>
       </c>
       <c r="AE16" t="inlineStr"/>
@@ -2540,44 +2558,46 @@
       <c r="AG16" t="inlineStr"/>
       <c r="AH16" t="inlineStr"/>
       <c r="AI16" t="inlineStr"/>
-      <c r="AJ16" t="inlineStr"/>
+      <c r="AJ16" t="n">
+        <v>50</v>
+      </c>
       <c r="AK16" t="inlineStr"/>
       <c r="AL16" t="inlineStr"/>
       <c r="AM16" t="n">
-        <v>564</v>
+        <v>144</v>
       </c>
       <c r="AN16" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="AO16" t="inlineStr"/>
       <c r="AP16" t="inlineStr"/>
       <c r="AQ16" t="n">
-        <v>0.06906</v>
+        <v>0.04783</v>
       </c>
       <c r="AR16" t="inlineStr"/>
       <c r="AS16" t="n">
-        <v>0.075</v>
+        <v>0.07439999999999999</v>
       </c>
       <c r="AT16" t="n">
-        <v>0.919</v>
+        <v>0.955</v>
       </c>
       <c r="AU16" t="n">
-        <v>0.881</v>
+        <v>0.95</v>
       </c>
       <c r="AV16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AW16" t="n">
-        <v>0.4384</v>
+        <v>0.3166</v>
       </c>
       <c r="AX16" t="n">
-        <v>2.2878</v>
+        <v>4.537</v>
       </c>
       <c r="AY16" t="n">
-        <v>0.1275</v>
+        <v>0.726</v>
       </c>
       <c r="AZ16" t="n">
-        <v>150</v>
+        <v>50</v>
       </c>
       <c r="BA16" t="inlineStr"/>
       <c r="BB16" t="inlineStr"/>
@@ -2590,64 +2610,40 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>EN_002</t>
+          <t>XGB_010</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Jonathan</t>
-        </is>
-      </c>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>ElasticNet</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>37</v>
-      </c>
-      <c r="F17" t="n">
-        <v>17</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="n">
         <v>5</v>
       </c>
-      <c r="H17" t="n">
-        <v>0.26348</v>
-      </c>
-      <c r="I17" t="n">
-        <v>176.6</v>
-      </c>
-      <c r="J17" t="n">
-        <v>0.29778</v>
-      </c>
-      <c r="K17" t="n">
-        <v>199.13</v>
-      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
-        <v>0.2815</v>
-      </c>
-      <c r="N17" t="n">
-        <v>313972117.03</v>
-      </c>
-      <c r="O17" t="n">
-        <v>1</v>
-      </c>
-      <c r="P17" t="n">
-        <v>0.01935773</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>1</v>
-      </c>
-      <c r="R17" t="n">
-        <v>0.00033828</v>
-      </c>
+        <v>0.13865</v>
+      </c>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr">
         <is>
           <t>5x5</t>
@@ -2655,48 +2651,84 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>submission_EN_002_l1r100_a2en02.csv</t>
+          <t>XGB_knn30_weighted_earlystop_XGB_010.csv</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>EN_002: log-transforms + interacciones + poly espacial. CV aleatorio MAE_log=0.26348 (optimista). CV espacial  MAE_log=0.29778 (honesto). Sesgo Δ=+0.03430. Modelo final: l1_ratio=1.0, α=1.94e-02. 17/37 coefs≠0.</t>
-        </is>
-      </c>
-      <c r="V17" t="n">
-        <v>0.0343</v>
-      </c>
+          <t>Base XGB_009 + precio ponderado por distancia K=30 vecinos. peso_i=1/dist_i (haversine km). LOO en train. Early stopping espacial. Sesgo Delta=+0.02231.</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr"/>
-      <c r="X17" t="inlineStr"/>
-      <c r="Y17" t="inlineStr"/>
-      <c r="Z17" t="inlineStr"/>
-      <c r="AA17" t="inlineStr"/>
+      <c r="X17" t="n">
+        <v>0.15029</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>0.00154</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>0.1726</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>0.00742</v>
+      </c>
       <c r="AB17" t="inlineStr"/>
       <c r="AC17" t="inlineStr"/>
-      <c r="AD17" t="inlineStr"/>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>structural=7, osm=10, text=11, geo=2 (lat+lon), precio_vecinos_ponderado=1 (K=30 LOO haversine), es_apartamento</t>
+        </is>
+      </c>
       <c r="AE17" t="inlineStr"/>
       <c r="AF17" t="inlineStr"/>
       <c r="AG17" t="inlineStr"/>
       <c r="AH17" t="inlineStr"/>
       <c r="AI17" t="inlineStr"/>
-      <c r="AJ17" t="inlineStr"/>
+      <c r="AJ17" t="n">
+        <v>50</v>
+      </c>
       <c r="AK17" t="inlineStr"/>
       <c r="AL17" t="inlineStr"/>
-      <c r="AM17" t="inlineStr"/>
-      <c r="AN17" t="inlineStr"/>
+      <c r="AM17" t="n">
+        <v>141</v>
+      </c>
+      <c r="AN17" t="n">
+        <v>8</v>
+      </c>
       <c r="AO17" t="inlineStr"/>
       <c r="AP17" t="inlineStr"/>
-      <c r="AQ17" t="inlineStr"/>
+      <c r="AQ17" t="n">
+        <v>0.02231</v>
+      </c>
       <c r="AR17" t="inlineStr"/>
-      <c r="AS17" t="inlineStr"/>
-      <c r="AT17" t="inlineStr"/>
-      <c r="AU17" t="inlineStr"/>
-      <c r="AV17" t="inlineStr"/>
-      <c r="AW17" t="inlineStr"/>
-      <c r="AX17" t="inlineStr"/>
-      <c r="AY17" t="inlineStr"/>
-      <c r="AZ17" t="inlineStr"/>
-      <c r="BA17" t="inlineStr"/>
+      <c r="AS17" t="n">
+        <v>0.0639</v>
+      </c>
+      <c r="AT17" t="n">
+        <v>0.998</v>
+      </c>
+      <c r="AU17" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="AV17" t="n">
+        <v>2</v>
+      </c>
+      <c r="AW17" t="n">
+        <v>0.4868</v>
+      </c>
+      <c r="AX17" t="n">
+        <v>2.5179</v>
+      </c>
+      <c r="AY17" t="n">
+        <v>0.4856</v>
+      </c>
+      <c r="AZ17" t="n">
+        <v>50</v>
+      </c>
+      <c r="BA17" t="n">
+        <v>30</v>
+      </c>
       <c r="BB17" t="inlineStr"/>
       <c r="BC17" t="inlineStr"/>
       <c r="BD17" t="inlineStr"/>
@@ -2707,32 +2739,30 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>NN_003</t>
+          <t>LR_001</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Jonathan</t>
+          <t>Natalia</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>NeuralNetwork_PyTorch</t>
+          <t>LinearRegression</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>val_split=0.2</t>
-        </is>
+      <c r="G18" t="n">
+        <v>5</v>
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
@@ -2740,11 +2770,9 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
-        <v>0.13739</v>
-      </c>
-      <c r="N18" t="n">
-        <v>216987903.08</v>
-      </c>
+        <v>0.27873</v>
+      </c>
+      <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
@@ -2756,61 +2784,45 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>submission_NN_003_ep182_p118k.csv</t>
+          <t>submission_LR_001_20260521.csv</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>NN_003: BN + 4 capas + features EN_002 + reg reducida + patience=30. Backend: mps. l1=5e-05, l2=5e-05. Épocas: 182/300. MAE_log val.interno=0.18910. MAE_log CV espacial=0.24331. Sesgo Δ=+0.05420.</t>
+          <t>OLS sin regularización. Baseline interpretable. CV aleatorio MAE_log=0.27905 (optimista). CV espacial  MAE_log=0.31016 (honesto). Sesgo Δ=+0.03111. 29 features (structural + text + osm + es_apartamento).</t>
         </is>
       </c>
       <c r="V18" t="inlineStr"/>
       <c r="W18" t="n">
-        <v>118145</v>
+        <v>30</v>
       </c>
       <c r="X18" t="n">
-        <v>0.1891</v>
-      </c>
-      <c r="Y18" t="inlineStr"/>
+        <v>0.27905</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>0.00197</v>
+      </c>
       <c r="Z18" t="n">
-        <v>0.24331</v>
-      </c>
-      <c r="AA18" t="inlineStr"/>
+        <v>0.31016</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>0.007849999999999999</v>
+      </c>
       <c r="AB18" t="inlineStr"/>
       <c r="AC18" t="inlineStr"/>
       <c r="AD18" t="inlineStr">
         <is>
-          <t>structural=10, text=11, osm=10, spatial_poly=5, es_apartamento</t>
-        </is>
-      </c>
-      <c r="AE18" t="n">
-        <v>182</v>
-      </c>
+          <t>structural=7, text=11, osm=10, es_apartamento</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr"/>
       <c r="AF18" t="inlineStr"/>
-      <c r="AG18" t="n">
-        <v>165.01</v>
-      </c>
-      <c r="AH18" t="inlineStr">
-        <is>
-          <t>p→256(BN,Drop0.2)→256(BN,Drop0.2)→128(BN,Drop0.1)→64(BN)→1 (ReLU)</t>
-        </is>
-      </c>
+      <c r="AG18" t="inlineStr"/>
+      <c r="AH18" t="inlineStr"/>
       <c r="AI18" t="inlineStr"/>
-      <c r="AJ18" t="inlineStr">
-        <is>
-          <t>patience=30</t>
-        </is>
-      </c>
-      <c r="AK18" t="inlineStr">
-        <is>
-          <t>l1=5e-05, l2=5e-05</t>
-        </is>
-      </c>
-      <c r="AL18" t="inlineStr">
-        <is>
-          <t>mps</t>
-        </is>
-      </c>
+      <c r="AJ18" t="inlineStr"/>
+      <c r="AK18" t="inlineStr"/>
+      <c r="AL18" t="inlineStr"/>
       <c r="AM18" t="inlineStr"/>
       <c r="AN18" t="inlineStr"/>
       <c r="AO18" t="inlineStr"/>
@@ -2836,40 +2848,62 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>XGB_007</t>
+          <t>EN_002</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Jonathan</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>ElasticNet</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>31</v>
-      </c>
-      <c r="F19" t="inlineStr"/>
+        <v>37</v>
+      </c>
+      <c r="F19" t="n">
+        <v>17</v>
+      </c>
       <c r="G19" t="n">
         <v>5</v>
       </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
+      <c r="H19" t="n">
+        <v>0.26348</v>
+      </c>
+      <c r="I19" t="n">
+        <v>176.6</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.29778</v>
+      </c>
+      <c r="K19" t="n">
+        <v>199.13</v>
+      </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
-        <v>0.17902</v>
+        <v>0.2815</v>
       </c>
       <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
+      <c r="O19" t="n">
+        <v>1</v>
+      </c>
+      <c r="P19" t="n">
+        <v>0.01935773</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>1</v>
+      </c>
+      <c r="R19" t="n">
+        <v>0.00033828</v>
+      </c>
       <c r="S19" t="inlineStr">
         <is>
           <t>5x5</t>
@@ -2877,81 +2911,47 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>XGB_latlon_earlystop_XGB_007.csv</t>
+          <t>submission_EN_002_l1r100_a2en02.csv</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>lat+lon como features geograficas directas. Early stopping=50 rondas. Mejor ronda=87. RandomizedSearch 50 iter. Sesgo Delta=+0.05153.</t>
-        </is>
-      </c>
-      <c r="V19" t="inlineStr"/>
+          <t>EN_002: log-transforms + interacciones + poly espacial. CV aleatorio MAE_log=0.26348 (optimista). CV espacial  MAE_log=0.29778 (honesto). Sesgo Δ=+0.03430. Modelo final: l1_ratio=1.0, α=1.94e-02. 17/37 coefs≠0.</t>
+        </is>
+      </c>
+      <c r="V19" t="n">
+        <v>0.0343</v>
+      </c>
       <c r="W19" t="inlineStr"/>
-      <c r="X19" t="n">
-        <v>0.17922</v>
-      </c>
-      <c r="Y19" t="n">
-        <v>0.00119</v>
-      </c>
-      <c r="Z19" t="n">
-        <v>0.23075</v>
-      </c>
-      <c r="AA19" t="n">
-        <v>0.00638</v>
-      </c>
+      <c r="X19" t="inlineStr"/>
+      <c r="Y19" t="inlineStr"/>
+      <c r="Z19" t="inlineStr"/>
+      <c r="AA19" t="inlineStr"/>
       <c r="AB19" t="inlineStr"/>
       <c r="AC19" t="inlineStr"/>
-      <c r="AD19" t="inlineStr">
-        <is>
-          <t>structural=7, osm=10, text=11, geo=2 (lat+lon), es_apartamento</t>
-        </is>
-      </c>
+      <c r="AD19" t="inlineStr"/>
       <c r="AE19" t="inlineStr"/>
       <c r="AF19" t="inlineStr"/>
       <c r="AG19" t="inlineStr"/>
       <c r="AH19" t="inlineStr"/>
       <c r="AI19" t="inlineStr"/>
-      <c r="AJ19" t="n">
-        <v>50</v>
-      </c>
+      <c r="AJ19" t="inlineStr"/>
       <c r="AK19" t="inlineStr"/>
       <c r="AL19" t="inlineStr"/>
-      <c r="AM19" t="n">
-        <v>87</v>
-      </c>
-      <c r="AN19" t="n">
-        <v>6</v>
-      </c>
+      <c r="AM19" t="inlineStr"/>
+      <c r="AN19" t="inlineStr"/>
       <c r="AO19" t="inlineStr"/>
       <c r="AP19" t="inlineStr"/>
-      <c r="AQ19" t="n">
-        <v>0.05153</v>
-      </c>
+      <c r="AQ19" t="inlineStr"/>
       <c r="AR19" t="inlineStr"/>
-      <c r="AS19" t="n">
-        <v>0.0742</v>
-      </c>
-      <c r="AT19" t="n">
-        <v>0.614</v>
-      </c>
-      <c r="AU19" t="n">
-        <v>0.898</v>
-      </c>
-      <c r="AV19" t="n">
-        <v>2</v>
-      </c>
-      <c r="AW19" t="n">
-        <v>0.445</v>
-      </c>
-      <c r="AX19" t="n">
-        <v>3.1023</v>
-      </c>
-      <c r="AY19" t="n">
-        <v>0.094</v>
-      </c>
-      <c r="AZ19" t="n">
-        <v>50</v>
-      </c>
+      <c r="AS19" t="inlineStr"/>
+      <c r="AT19" t="inlineStr"/>
+      <c r="AU19" t="inlineStr"/>
+      <c r="AV19" t="inlineStr"/>
+      <c r="AW19" t="inlineStr"/>
+      <c r="AX19" t="inlineStr"/>
+      <c r="AY19" t="inlineStr"/>
+      <c r="AZ19" t="inlineStr"/>
       <c r="BA19" t="inlineStr"/>
       <c r="BB19" t="inlineStr"/>
       <c r="BC19" t="inlineStr"/>
@@ -2963,22 +2963,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>XGB_008</t>
+          <t>CART_002</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>CART</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="n">
@@ -2990,7 +2990,7 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
-        <v>0.17408</v>
+        <v>0.22825</v>
       </c>
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
@@ -3004,33 +3004,33 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>XGB_filtro_chapinero_earlystop_XGB_008.csv</t>
+          <t>CART_d10_leaf20_ccp00001_cv5_CART_002.csv</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>Filtro train por rango IQR precio_m2 de Chapinero. Train: 38644 -&gt; 37918 obs. Rango: [-1,767,548, 12,489,100] COP/m2. Early stopping=50, mejor ronda=144. Sesgo Delta=+0.04783.</t>
+          <t>All features: estructurales + OSM + texto. GridSearchCV espacial. Params: {'ccp_alpha': 0.0001, 'max_depth': 10, 'min_samples_leaf': 20}. Sesgo Delta=+0.04144.</t>
         </is>
       </c>
       <c r="V20" t="inlineStr"/>
       <c r="W20" t="inlineStr"/>
       <c r="X20" t="n">
-        <v>0.17798</v>
+        <v>0.2326</v>
       </c>
       <c r="Y20" t="n">
-        <v>0.00256</v>
+        <v>0.00216</v>
       </c>
       <c r="Z20" t="n">
-        <v>0.22582</v>
+        <v>0.27405</v>
       </c>
       <c r="AA20" t="n">
-        <v>0.01073</v>
+        <v>0.01087</v>
       </c>
       <c r="AB20" t="inlineStr"/>
       <c r="AC20" t="inlineStr"/>
       <c r="AD20" t="inlineStr">
         <is>
-          <t>structural=7, osm=10, text=11, geo=2 (lat+lon), es_apartamento</t>
+          <t>structural=7, osm=10, text=11, es_apartamento</t>
         </is>
       </c>
       <c r="AE20" t="inlineStr"/>
@@ -3038,47 +3038,31 @@
       <c r="AG20" t="inlineStr"/>
       <c r="AH20" t="inlineStr"/>
       <c r="AI20" t="inlineStr"/>
-      <c r="AJ20" t="n">
-        <v>50</v>
-      </c>
+      <c r="AJ20" t="inlineStr"/>
       <c r="AK20" t="inlineStr"/>
       <c r="AL20" t="inlineStr"/>
-      <c r="AM20" t="n">
-        <v>144</v>
-      </c>
+      <c r="AM20" t="inlineStr"/>
       <c r="AN20" t="n">
-        <v>5</v>
-      </c>
-      <c r="AO20" t="inlineStr"/>
+        <v>10</v>
+      </c>
+      <c r="AO20" t="n">
+        <v>20</v>
+      </c>
       <c r="AP20" t="inlineStr"/>
       <c r="AQ20" t="n">
-        <v>0.04783</v>
-      </c>
-      <c r="AR20" t="inlineStr"/>
-      <c r="AS20" t="n">
-        <v>0.07439999999999999</v>
-      </c>
-      <c r="AT20" t="n">
-        <v>0.955</v>
-      </c>
-      <c r="AU20" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="AV20" t="n">
-        <v>3</v>
-      </c>
-      <c r="AW20" t="n">
-        <v>0.3166</v>
-      </c>
-      <c r="AX20" t="n">
-        <v>4.537</v>
-      </c>
-      <c r="AY20" t="n">
-        <v>0.726</v>
-      </c>
-      <c r="AZ20" t="n">
-        <v>50</v>
-      </c>
+        <v>0.04144</v>
+      </c>
+      <c r="AR20" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="AS20" t="inlineStr"/>
+      <c r="AT20" t="inlineStr"/>
+      <c r="AU20" t="inlineStr"/>
+      <c r="AV20" t="inlineStr"/>
+      <c r="AW20" t="inlineStr"/>
+      <c r="AX20" t="inlineStr"/>
+      <c r="AY20" t="inlineStr"/>
+      <c r="AZ20" t="inlineStr"/>
       <c r="BA20" t="inlineStr"/>
       <c r="BB20" t="inlineStr"/>
       <c r="BC20" t="inlineStr"/>
@@ -3090,22 +3074,26 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>XGB_009</t>
+          <t>RF_005</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="n">
@@ -3117,7 +3105,7 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
-        <v>0.16854</v>
+        <v>0.16414</v>
       </c>
       <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
@@ -3131,33 +3119,33 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>XGB_knn30_latlon_earlystop_XGB_009.csv</t>
+          <t>RF_ntrees500_d15_leaf5_mfsqrt_cv5_gridESP_RF_005.csv</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>Base XGB_007 + precio mediano K=30 vecinos (haversine, LOO). Early stopping espacial bloque mas grande. Sesgo Delta=+0.03480.</t>
+          <t>Grid search max_depth=[8, 10, 15] via CV espacial. Best depth=15. n_estimators=500, min_samples_leaf=5. Features completas. Sesgo Δ=+0.07192.</t>
         </is>
       </c>
       <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr"/>
       <c r="X21" t="n">
-        <v>0.17598</v>
+        <v>0.19172</v>
       </c>
       <c r="Y21" t="n">
-        <v>0.0016</v>
+        <v>0.00195</v>
       </c>
       <c r="Z21" t="n">
-        <v>0.21079</v>
+        <v>0.26364</v>
       </c>
       <c r="AA21" t="n">
-        <v>0.00991</v>
+        <v>0.00848</v>
       </c>
       <c r="AB21" t="inlineStr"/>
       <c r="AC21" t="inlineStr"/>
       <c r="AD21" t="inlineStr">
         <is>
-          <t>structural=7, osm=10, text=11, geo=2 (lat+lon), precio_vecinos=1 (K=30 LOO), es_apartamento</t>
+          <t>structural=7, text=11, osm=10, es_apartamento</t>
         </is>
       </c>
       <c r="AE21" t="inlineStr"/>
@@ -3165,50 +3153,36 @@
       <c r="AG21" t="inlineStr"/>
       <c r="AH21" t="inlineStr"/>
       <c r="AI21" t="inlineStr"/>
-      <c r="AJ21" t="n">
-        <v>50</v>
-      </c>
+      <c r="AJ21" t="inlineStr"/>
       <c r="AK21" t="inlineStr"/>
       <c r="AL21" t="inlineStr"/>
       <c r="AM21" t="n">
-        <v>265</v>
+        <v>500</v>
       </c>
       <c r="AN21" t="n">
-        <v>6</v>
-      </c>
-      <c r="AO21" t="inlineStr"/>
-      <c r="AP21" t="inlineStr"/>
+        <v>15</v>
+      </c>
+      <c r="AO21" t="n">
+        <v>5</v>
+      </c>
+      <c r="AP21" t="inlineStr">
+        <is>
+          <t>sqrt</t>
+        </is>
+      </c>
       <c r="AQ21" t="n">
-        <v>0.0348</v>
+        <v>0.07192</v>
       </c>
       <c r="AR21" t="inlineStr"/>
-      <c r="AS21" t="n">
-        <v>0.026</v>
-      </c>
-      <c r="AT21" t="n">
-        <v>0.749</v>
-      </c>
-      <c r="AU21" t="n">
-        <v>0.89</v>
-      </c>
-      <c r="AV21" t="n">
-        <v>6</v>
-      </c>
-      <c r="AW21" t="n">
-        <v>0.321</v>
-      </c>
-      <c r="AX21" t="n">
-        <v>3.1131</v>
-      </c>
-      <c r="AY21" t="n">
-        <v>0.669</v>
-      </c>
-      <c r="AZ21" t="n">
-        <v>50</v>
-      </c>
-      <c r="BA21" t="n">
-        <v>30</v>
-      </c>
+      <c r="AS21" t="inlineStr"/>
+      <c r="AT21" t="inlineStr"/>
+      <c r="AU21" t="inlineStr"/>
+      <c r="AV21" t="inlineStr"/>
+      <c r="AW21" t="inlineStr"/>
+      <c r="AX21" t="inlineStr"/>
+      <c r="AY21" t="inlineStr"/>
+      <c r="AZ21" t="inlineStr"/>
+      <c r="BA21" t="inlineStr"/>
       <c r="BB21" t="inlineStr"/>
       <c r="BC21" t="inlineStr"/>
       <c r="BD21" t="inlineStr"/>
@@ -3219,12 +3193,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>XGB_010</t>
+          <t>XGB_009</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -3246,7 +3220,7 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
-        <v>0.13865</v>
+        <v>0.16854</v>
       </c>
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
@@ -3260,33 +3234,33 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>XGB_knn30_weighted_earlystop_XGB_010.csv</t>
+          <t>XGB_knn30_latlon_earlystop_XGB_009.csv</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>Base XGB_009 + precio ponderado por distancia K=30 vecinos. peso_i=1/dist_i (haversine km). LOO en train. Early stopping espacial. Sesgo Delta=+0.02231.</t>
+          <t>Base XGB_007 + precio mediano K=30 vecinos (haversine, LOO). Early stopping espacial bloque mas grande. Sesgo Delta=+0.03480.</t>
         </is>
       </c>
       <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr"/>
       <c r="X22" t="n">
-        <v>0.15029</v>
+        <v>0.17598</v>
       </c>
       <c r="Y22" t="n">
-        <v>0.00154</v>
+        <v>0.0016</v>
       </c>
       <c r="Z22" t="n">
-        <v>0.1726</v>
+        <v>0.21079</v>
       </c>
       <c r="AA22" t="n">
-        <v>0.00742</v>
+        <v>0.00991</v>
       </c>
       <c r="AB22" t="inlineStr"/>
       <c r="AC22" t="inlineStr"/>
       <c r="AD22" t="inlineStr">
         <is>
-          <t>structural=7, osm=10, text=11, geo=2 (lat+lon), precio_vecinos_ponderado=1 (K=30 LOO haversine), es_apartamento</t>
+          <t>structural=7, osm=10, text=11, geo=2 (lat+lon), precio_vecinos=1 (K=30 LOO), es_apartamento</t>
         </is>
       </c>
       <c r="AE22" t="inlineStr"/>
@@ -3300,37 +3274,37 @@
       <c r="AK22" t="inlineStr"/>
       <c r="AL22" t="inlineStr"/>
       <c r="AM22" t="n">
-        <v>141</v>
+        <v>265</v>
       </c>
       <c r="AN22" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AO22" t="inlineStr"/>
       <c r="AP22" t="inlineStr"/>
       <c r="AQ22" t="n">
-        <v>0.02231</v>
+        <v>0.0348</v>
       </c>
       <c r="AR22" t="inlineStr"/>
       <c r="AS22" t="n">
-        <v>0.0639</v>
+        <v>0.026</v>
       </c>
       <c r="AT22" t="n">
-        <v>0.998</v>
+        <v>0.749</v>
       </c>
       <c r="AU22" t="n">
-        <v>0.97</v>
+        <v>0.89</v>
       </c>
       <c r="AV22" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AW22" t="n">
-        <v>0.4868</v>
+        <v>0.321</v>
       </c>
       <c r="AX22" t="n">
-        <v>2.5179</v>
+        <v>3.1131</v>
       </c>
       <c r="AY22" t="n">
-        <v>0.4856</v>
+        <v>0.669</v>
       </c>
       <c r="AZ22" t="n">
         <v>50</v>
@@ -3348,80 +3322,108 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SL_003</t>
+          <t>NN_003</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Equipo</t>
+          <t>Jonathan</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>SuperLearner</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr"/>
+          <t>NeuralNetwork_PyTorch</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>37</v>
+      </c>
       <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>val_split=0.2</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
-        <v>0.146442</v>
-      </c>
-      <c r="N23" t="n">
-        <v>199851631.65</v>
-      </c>
+        <v>0.1504</v>
+      </c>
+      <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>5x5</t>
+        </is>
+      </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>submission_SL_003_20260520.csv</t>
+          <t>submission_NN_003_ep133_p118k.csv</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>Ganador: SL-2 (SL-2 MAE_esp=0.23244 vs SL-3 MAE_esp=0.23123). Meta: NNLS (positive=True). Pesos: [XGB_009:0.580 | NN_003:0.454]. Bases: XGB_009 (KNN K=30 LOO) + NN_003 (PyTorch 256x256x128x64). CV 5-fold + espacial 5x5. Δ=+0.06700.</t>
-        </is>
-      </c>
-      <c r="V23" t="n">
-        <v>0.066996</v>
-      </c>
-      <c r="W23" t="inlineStr"/>
+          <t>NN_003: BN + 4 capas + features EN_002 + reg reducida + patience=30. Backend: mps. l1=5e-05, l2=5e-05. Épocas: 133/300. MAE_log val.interno=0.19135. MAE_log CV espacial=0.23926. Sesgo Δ=+0.04791.</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr"/>
+      <c r="W23" t="n">
+        <v>118145</v>
+      </c>
       <c r="X23" t="n">
-        <v>0.165447</v>
-      </c>
-      <c r="Y23" t="n">
-        <v>0.002361</v>
-      </c>
+        <v>0.19135</v>
+      </c>
+      <c r="Y23" t="inlineStr"/>
       <c r="Z23" t="n">
-        <v>0.232444</v>
-      </c>
-      <c r="AA23" t="n">
-        <v>0.008907999999999999</v>
-      </c>
+        <v>0.23926</v>
+      </c>
+      <c r="AA23" t="inlineStr"/>
       <c r="AB23" t="inlineStr"/>
       <c r="AC23" t="inlineStr"/>
-      <c r="AD23" t="inlineStr"/>
-      <c r="AE23" t="inlineStr"/>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>structural=10, text=11, osm=10, spatial_poly=5, es_apartamento</t>
+        </is>
+      </c>
+      <c r="AE23" t="n">
+        <v>133</v>
+      </c>
       <c r="AF23" t="inlineStr"/>
-      <c r="AG23" t="inlineStr"/>
-      <c r="AH23" t="inlineStr"/>
+      <c r="AG23" t="n">
+        <v>161.51</v>
+      </c>
+      <c r="AH23" t="inlineStr">
+        <is>
+          <t>p→256(BN,Drop0.2)→256(BN,Drop0.2)→128(BN,Drop0.1)→64(BN)→1 (ReLU)</t>
+        </is>
+      </c>
       <c r="AI23" t="inlineStr"/>
-      <c r="AJ23" t="inlineStr"/>
-      <c r="AK23" t="inlineStr"/>
-      <c r="AL23" t="inlineStr"/>
+      <c r="AJ23" t="inlineStr">
+        <is>
+          <t>patience=30</t>
+        </is>
+      </c>
+      <c r="AK23" t="inlineStr">
+        <is>
+          <t>l1=5e-05, l2=5e-05</t>
+        </is>
+      </c>
+      <c r="AL23" t="inlineStr">
+        <is>
+          <t>mps</t>
+        </is>
+      </c>
       <c r="AM23" t="inlineStr"/>
       <c r="AN23" t="inlineStr"/>
       <c r="AO23" t="inlineStr"/>
@@ -3437,29 +3439,17 @@
       <c r="AY23" t="inlineStr"/>
       <c r="AZ23" t="inlineStr"/>
       <c r="BA23" t="inlineStr"/>
-      <c r="BB23" t="n">
-        <v>0.165447</v>
-      </c>
-      <c r="BC23" t="n">
-        <v>0.002361</v>
-      </c>
-      <c r="BD23" t="n">
-        <v>0.232444</v>
-      </c>
-      <c r="BE23" t="n">
-        <v>0.008907999999999999</v>
-      </c>
-      <c r="BF23" t="n">
-        <v>0.146442</v>
-      </c>
-      <c r="BG23" t="n">
-        <v>0.066996</v>
-      </c>
+      <c r="BB23" t="inlineStr"/>
+      <c r="BC23" t="inlineStr"/>
+      <c r="BD23" t="inlineStr"/>
+      <c r="BE23" t="inlineStr"/>
+      <c r="BF23" t="inlineStr"/>
+      <c r="BG23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>LR_001</t>
+          <t>SL_003</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3469,72 +3459,62 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Natalia</t>
+          <t>Equipo</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>LinearRegression</t>
+          <t>SuperLearner</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>29</v>
+        <v>69</v>
       </c>
       <c r="F24" t="inlineStr"/>
-      <c r="G24" t="n">
-        <v>5</v>
-      </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
-        <v>0.27873</v>
+        <v>0.143768</v>
       </c>
       <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t>5x5</t>
-        </is>
-      </c>
+      <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>submission_LR_001_20260521.csv</t>
+          <t>submission_SL_003_20260521.csv</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>OLS sin regularización. Baseline interpretable. CV aleatorio MAE_log=0.27905 (optimista). CV espacial  MAE_log=0.31016 (honesto). Sesgo Δ=+0.03111. 29 features (structural + text + osm + es_apartamento).</t>
-        </is>
-      </c>
-      <c r="V24" t="inlineStr"/>
-      <c r="W24" t="n">
-        <v>30</v>
-      </c>
+          <t>Ganador: SL-2 (SL-2 esp=0.23350 vs SL-3 esp=0.23228). Meta: NNLS (positive=True). Pesos: [XGB_009:0.584 | NN_003:0.458]. Bases: XGB_009 (KNN K=30 LOO) + NN_003 (PyTorch 256x256x128x64). CV 5-fold + espacial 5x5. Δ=+0.06781.</t>
+        </is>
+      </c>
+      <c r="V24" t="n">
+        <v>0.067811</v>
+      </c>
+      <c r="W24" t="inlineStr"/>
       <c r="X24" t="n">
-        <v>0.27905</v>
+        <v>0.165691</v>
       </c>
       <c r="Y24" t="n">
-        <v>0.00197</v>
+        <v>0.001995</v>
       </c>
       <c r="Z24" t="n">
-        <v>0.31016</v>
+        <v>0.233501</v>
       </c>
       <c r="AA24" t="n">
-        <v>0.007849999999999999</v>
+        <v>0.009377</v>
       </c>
       <c r="AB24" t="inlineStr"/>
       <c r="AC24" t="inlineStr"/>
-      <c r="AD24" t="inlineStr">
-        <is>
-          <t>structural=7, text=11, osm=10, es_apartamento</t>
-        </is>
-      </c>
+      <c r="AD24" t="inlineStr"/>
       <c r="AE24" t="inlineStr"/>
       <c r="AF24" t="inlineStr"/>
       <c r="AG24" t="inlineStr"/>

</xml_diff>